<commit_message>
ODK: translate only the form's breed choices, and reject future resolution dates
The ingest hooks mapped a breed by substring and, when nothing matched, to
the "local" breed of the animal's species, so a goat breed on a cattle row,
or a typo, was silently stored as Local Zebu. Breeds are now translated
through an exact map of the form's 46 choices per species; anything else is
passed through unchanged for domain validation to reject. test_transform.py
checks that every choice in odk/breed_choices.csv maps to a breed of its own
species in the code list.

Form v4 (published on the dev Central) adds "not in the future" to the
health-event and vital-event resolution dates.
</commit_message>
<xml_diff>
--- a/odk/livestock_registry.xlsx
+++ b/odk/livestock_registry.xlsx
@@ -1689,12 +1689,12 @@
       </c>
       <c r="J44" s="15" t="inlineStr">
         <is>
-          <t>. &gt;= ${date_onset} or ${date_onset} = ''</t>
+          <t>(. &gt;= ${date_onset} or ${date_onset} = '') and . &lt;= today()</t>
         </is>
       </c>
       <c r="K44" s="15" t="inlineStr">
         <is>
-          <t>Resolution date must be on or after onset date</t>
+          <t>Resolution date must be on or after the onset date and not in the future</t>
         </is>
       </c>
     </row>
@@ -2455,12 +2455,12 @@
       </c>
       <c r="J77" s="15" t="inlineStr">
         <is>
-          <t>. &gt;= ${vital_date_onset} or ${vital_date_onset} = ''</t>
+          <t>(. &gt;= ${vital_date_onset} or ${vital_date_onset} = '') and . &lt;= today()</t>
         </is>
       </c>
       <c r="K77" s="15" t="inlineStr">
         <is>
-          <t>Resolution date must be on or after onset date</t>
+          <t>Resolution date must be on or after the onset date and not in the future</t>
         </is>
       </c>
     </row>
@@ -3269,7 +3269,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="13.5" customHeight="1" s="18">
       <c r="A13" s="15" t="inlineStr">
         <is>
@@ -4282,7 +4281,6 @@
         </is>
       </c>
     </row>
-    <row r="59"/>
     <row r="60" ht="13.5" customHeight="1" s="18">
       <c r="A60" s="15" t="inlineStr">
         <is>
@@ -4334,7 +4332,6 @@
         </is>
       </c>
     </row>
-    <row r="63"/>
     <row r="64" ht="13.5" customHeight="1" s="18">
       <c r="A64" s="15" t="inlineStr">
         <is>
@@ -4403,7 +4400,6 @@
         </is>
       </c>
     </row>
-    <row r="68"/>
     <row r="69" ht="13.5" customHeight="1" s="18">
       <c r="A69" s="15" t="inlineStr">
         <is>
@@ -4455,7 +4451,6 @@
         </is>
       </c>
     </row>
-    <row r="72"/>
     <row r="73" ht="13.5" customHeight="1" s="18">
       <c r="A73" s="15" t="inlineStr">
         <is>
@@ -4524,7 +4519,6 @@
         </is>
       </c>
     </row>
-    <row r="77"/>
     <row r="78" ht="13.5" customHeight="1" s="18">
       <c r="A78" s="15" t="inlineStr">
         <is>
@@ -4559,7 +4553,6 @@
         </is>
       </c>
     </row>
-    <row r="80"/>
     <row r="81" ht="13.5" customHeight="1" s="18">
       <c r="A81" s="15" t="inlineStr">
         <is>
@@ -4611,7 +4604,6 @@
         </is>
       </c>
     </row>
-    <row r="84"/>
     <row r="85" ht="13.5" customHeight="1" s="18">
       <c r="A85" s="15" t="inlineStr">
         <is>
@@ -4732,7 +4724,6 @@
         </is>
       </c>
     </row>
-    <row r="93"/>
     <row r="94" ht="13.5" customHeight="1" s="18">
       <c r="A94" s="15" t="inlineStr">
         <is>
@@ -4835,7 +4826,6 @@
         </is>
       </c>
     </row>
-    <row r="100"/>
     <row r="101" ht="13.5" customHeight="1" s="18">
       <c r="A101" s="15" t="inlineStr">
         <is>
@@ -5386,8 +5376,6 @@
         </is>
       </c>
     </row>
-    <row r="126"/>
-    <row r="127"/>
     <row r="128" ht="13.5" customHeight="1" s="18">
       <c r="A128" s="15" t="inlineStr">
         <is>
@@ -5422,7 +5410,6 @@
         </is>
       </c>
     </row>
-    <row r="130"/>
     <row r="131" ht="13.5" customHeight="1" s="18">
       <c r="A131" s="15" t="inlineStr">
         <is>
@@ -5474,7 +5461,6 @@
         </is>
       </c>
     </row>
-    <row r="134"/>
     <row r="135" ht="13.5" customHeight="1" s="18">
       <c r="A135" s="15" t="inlineStr">
         <is>
@@ -5917,7 +5903,6 @@
         </is>
       </c>
     </row>
-    <row r="161"/>
     <row r="162" ht="13.5" customHeight="1" s="18">
       <c r="A162" s="15" t="inlineStr">
         <is>
@@ -6094,7 +6079,7 @@
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v4</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Make every ODK form text readable: required messages, plain validation messages and hints
Field names, choice names, constraints and calculations are unchanged. Form
version v5.
</commit_message>
<xml_diff>
--- a/odk/livestock_registry.xlsx
+++ b/odk/livestock_registry.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M106"/>
+  <dimension ref="A1:N106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.4765625" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26.36" customWidth="1" style="15" min="1" max="1"/>
@@ -498,6 +498,11 @@
           <t>choice_filter</t>
         </is>
       </c>
+      <c r="N1" s="15" t="inlineStr">
+        <is>
+          <t>required_message</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="13.5" customHeight="1" s="18">
       <c r="A2" s="15" t="inlineStr">
@@ -558,7 +563,7 @@
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Optional. Format: FR- followed by 10 digits (e.g. FR-1234567890)</t>
+          <t>Optional. FR- followed by 10 digits, for example FR-1234567890.</t>
         </is>
       </c>
       <c r="J5" s="15" t="inlineStr">
@@ -568,7 +573,7 @@
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
-          <t>farmer_id must be FR- followed by exactly 10 digits</t>
+          <t>The Farmer ID must be FR- followed by exactly 10 digits, for example FR-1234567890.</t>
         </is>
       </c>
     </row>
@@ -585,12 +590,12 @@
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>Fayda FAN ID</t>
+          <t>Fayda FAN (16-digit Fayda number)</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>Format: exactly 16 digits</t>
+          <t>The 16-digit Fayda number, digits only.</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
@@ -607,11 +612,16 @@
       </c>
       <c r="K6" s="21" t="inlineStr">
         <is>
-          <t>Fayda ID must contain exactly 16 digits.</t>
+          <t>Enter the 16-digit Fayda number, using digits only.</t>
         </is>
       </c>
       <c r="L6" s="20" t="n"/>
       <c r="M6" s="20" t="n"/>
+      <c r="N6" s="15" t="inlineStr">
+        <is>
+          <t>Enter the 16-digit Fayda number.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customFormat="1" customHeight="1" s="15">
       <c r="A7" s="20" t="inlineStr">
@@ -641,6 +651,11 @@
       <c r="K7" s="23" t="n"/>
       <c r="L7" s="20" t="n"/>
       <c r="M7" s="20" t="n"/>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>Enter the first name.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customFormat="1" customHeight="1" s="15">
       <c r="A8" s="20" t="inlineStr">
@@ -688,6 +703,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Enter the last name.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="13.5" customHeight="1" s="18">
       <c r="A10" s="15" t="inlineStr">
@@ -729,7 +749,7 @@
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>Date of birth must not be in the future</t>
+          <t>The date of birth cannot be in the future.</t>
         </is>
       </c>
     </row>
@@ -751,7 +771,7 @@
       </c>
       <c r="D12" s="21" t="inlineStr">
         <is>
-          <t>Format: 0911223344 or +251911223344</t>
+          <t>For example 0911223344 or +251911223344.</t>
         </is>
       </c>
       <c r="I12" s="15" t="inlineStr">
@@ -766,7 +786,7 @@
       </c>
       <c r="K12" s="21" t="inlineStr">
         <is>
-          <t>Enter valid Ethiopian number: 0911223344 or +251911223344</t>
+          <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
     </row>
@@ -803,12 +823,17 @@
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>Registration date must not be in the future</t>
+          <t>The registration date cannot be in the future.</t>
         </is>
       </c>
       <c r="L13" s="15" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Enter the registration date.</t>
         </is>
       </c>
     </row>
@@ -862,7 +887,7 @@
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>DA Name</t>
+          <t>Development Agent Name</t>
         </is>
       </c>
       <c r="D16" s="20" t="n"/>
@@ -888,12 +913,12 @@
       </c>
       <c r="C17" s="20" t="inlineStr">
         <is>
-          <t>DA Mobile Number</t>
+          <t>Development Agent Mobile Number</t>
         </is>
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
-          <t>Format: 0911223344 or +251911223344</t>
+          <t>For example 0911223344 or +251911223344.</t>
         </is>
       </c>
       <c r="E17" s="20" t="n"/>
@@ -910,7 +935,7 @@
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
-          <t>Enter valid Ethiopian number: 0911223344 or +251911223344</t>
+          <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
       <c r="L17" s="20" t="n"/>
@@ -959,7 +984,7 @@
       </c>
       <c r="D19" s="21" t="inlineStr">
         <is>
-          <t>Format: 0911223344 or +251911223344</t>
+          <t>For example 0911223344 or +251911223344.</t>
         </is>
       </c>
       <c r="E19" s="20" t="n"/>
@@ -976,7 +1001,7 @@
       </c>
       <c r="K19" s="21" t="inlineStr">
         <is>
-          <t>Enter valid Ethiopian number: 0911223344 or +251911223344</t>
+          <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
       <c r="L19" s="20" t="n"/>
@@ -1182,6 +1207,11 @@
         </is>
       </c>
       <c r="J28" s="21" t="n"/>
+      <c r="N28" s="15" t="inlineStr">
+        <is>
+          <t>Select the species.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1" s="18">
       <c r="A29" s="15" t="inlineStr">
@@ -1216,6 +1246,11 @@
           <t>species = ${species_id}</t>
         </is>
       </c>
+      <c r="N29" s="15" t="inlineStr">
+        <is>
+          <t>Select the breed.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="18">
       <c r="A30" s="15" t="inlineStr">
@@ -1235,7 +1270,7 @@
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>Ear tag ID must be in format ET0000000000</t>
+          <t>ET followed by 10 digits, for example ET0123456789.</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
@@ -1255,7 +1290,12 @@
       </c>
       <c r="K30" s="15" t="inlineStr">
         <is>
-          <t>Ear tag must be ET + 10 digits (e.g. ET0000000000) and must not be repeated in this record</t>
+          <t>Enter the ear tag as ET followed by 10 digits, for example ET0123456789. Each animal in this record needs a different ear tag.</t>
+        </is>
+      </c>
+      <c r="N30" s="15" t="inlineStr">
+        <is>
+          <t>Enter the livestock ear tag.</t>
         </is>
       </c>
     </row>
@@ -1292,10 +1332,15 @@
       </c>
       <c r="K31" s="15" t="inlineStr">
         <is>
-          <t>This secondary identifier is used more than once in this record</t>
+          <t>This identifier is already used by another animal in this record. Enter a different one.</t>
         </is>
       </c>
       <c r="M31" s="21" t="n"/>
+      <c r="N31" s="15" t="inlineStr">
+        <is>
+          <t>Enter the secondary identifier (leg band / wing tag / hive number).</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="30" customHeight="1" s="18">
       <c r="A32" s="15" t="inlineStr">
@@ -1310,7 +1355,7 @@
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Quantity (Head Count)</t>
+          <t>Number of Animals or Hives</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
@@ -1330,10 +1375,15 @@
       </c>
       <c r="K32" s="15" t="inlineStr">
         <is>
-          <t>Quantity must be greater than 0</t>
+          <t>Enter a number greater than 0.</t>
         </is>
       </c>
       <c r="M32" s="21" t="n"/>
+      <c r="N32" s="15" t="inlineStr">
+        <is>
+          <t>Enter the number of animals or hives.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="13.5" customHeight="1" s="18">
       <c r="A33" s="15" t="inlineStr">
@@ -1358,7 +1408,7 @@
       </c>
       <c r="K33" s="15" t="inlineStr">
         <is>
-          <t>Weight must be greater than 0</t>
+          <t>Enter a weight greater than 0 kg.</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1445,12 @@
       </c>
       <c r="K34" s="15" t="inlineStr">
         <is>
-          <t>Date of birth must not be in the future</t>
+          <t>The date of birth cannot be in the future.</t>
+        </is>
+      </c>
+      <c r="N34" s="15" t="inlineStr">
+        <is>
+          <t>Enter the date of birth.</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1482,12 @@
       </c>
       <c r="K35" s="15" t="inlineStr">
         <is>
-          <t>'Mixed / Not Applicable' is allowed only for poultry and beehive</t>
+          <t>Mixed / Not Applicable can only be chosen for poultry and beehives. Choose Male or Female.</t>
+        </is>
+      </c>
+      <c r="N35" s="15" t="inlineStr">
+        <is>
+          <t>Select the sex.</t>
         </is>
       </c>
     </row>
@@ -1462,6 +1522,11 @@
           <t>minimal</t>
         </is>
       </c>
+      <c r="N36" s="15" t="inlineStr">
+        <is>
+          <t>Select the health status.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="13.5" customHeight="1" s="18">
       <c r="A37" s="15" t="inlineStr">
@@ -1494,6 +1559,11 @@
           <t>minimal</t>
         </is>
       </c>
+      <c r="N37" s="15" t="inlineStr">
+        <is>
+          <t>Select the vaccination status.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="13.5" customHeight="1" s="18">
       <c r="A38" s="15" t="inlineStr">
@@ -1528,12 +1598,17 @@
       </c>
       <c r="K38" s="15" t="inlineStr">
         <is>
-          <t>Registration date must not be in the future</t>
+          <t>The registration date cannot be in the future.</t>
         </is>
       </c>
       <c r="L38" s="15" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="N38" s="15" t="inlineStr">
+        <is>
+          <t>Enter the registration date.</t>
         </is>
       </c>
     </row>
@@ -1591,6 +1666,11 @@
           <t>minimal</t>
         </is>
       </c>
+      <c r="N41" s="15" t="inlineStr">
+        <is>
+          <t>Select the event type.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="18">
       <c r="A42" s="15" t="inlineStr">
@@ -1623,6 +1703,11 @@
           <t>minimal</t>
         </is>
       </c>
+      <c r="N42" s="15" t="inlineStr">
+        <is>
+          <t>Select the disease.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1" s="18">
       <c r="A43" s="15" t="inlineStr">
@@ -1657,7 +1742,12 @@
       </c>
       <c r="K43" s="15" t="inlineStr">
         <is>
-          <t>Onset date must not be in the future, and this event (same type and onset date) is already entered for this animal</t>
+          <t>The onset date cannot be in the future, and the same event with the same onset date cannot be entered twice for one animal.</t>
+        </is>
+      </c>
+      <c r="N43" s="15" t="inlineStr">
+        <is>
+          <t>Enter the date of onset.</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1784,12 @@
       </c>
       <c r="K44" s="15" t="inlineStr">
         <is>
-          <t>Resolution date must be on or after the onset date and not in the future</t>
+          <t>The resolution date must be on or after the onset date and cannot be in the future.</t>
+        </is>
+      </c>
+      <c r="N44" s="15" t="inlineStr">
+        <is>
+          <t>Enter the date of resolution.</t>
         </is>
       </c>
     </row>
@@ -1714,6 +1809,11 @@
           <t>Notifiable Disease</t>
         </is>
       </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
+        </is>
+      </c>
       <c r="F45" s="15" t="inlineStr">
         <is>
           <t>no</t>
@@ -1814,7 +1914,7 @@
       </c>
       <c r="D49" s="15" t="inlineStr">
         <is>
-          <t>e.g. exact address, clinic name</t>
+          <t>For example the exact address or the clinic name.</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1936,7 @@
       </c>
       <c r="D50" s="15" t="inlineStr">
         <is>
-          <t>Additional notes…</t>
+          <t>Any additional notes.</t>
         </is>
       </c>
       <c r="E50" s="15" t="n"/>
@@ -1919,6 +2019,11 @@
           <t>species = ${species_id}</t>
         </is>
       </c>
+      <c r="N54" s="15" t="inlineStr">
+        <is>
+          <t>Select the vaccine.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="13.5" customHeight="1" s="18">
       <c r="A55" s="15" t="inlineStr">
@@ -1953,7 +2058,12 @@
       </c>
       <c r="K55" s="15" t="inlineStr">
         <is>
-          <t>Vaccination date must not be in the future, and this vaccine on this date is already entered for this animal</t>
+          <t>The vaccination date cannot be in the future, and the same vaccine with the same date cannot be entered twice for one animal.</t>
+        </is>
+      </c>
+      <c r="N55" s="15" t="inlineStr">
+        <is>
+          <t>Enter the vaccination date.</t>
         </is>
       </c>
     </row>
@@ -1980,7 +2090,7 @@
       </c>
       <c r="K56" s="15" t="inlineStr">
         <is>
-          <t>Next due date must not be before the vaccination date</t>
+          <t>The next due date cannot be before the vaccination date.</t>
         </is>
       </c>
     </row>
@@ -1997,7 +2107,7 @@
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>Batch/Lot Number</t>
+          <t>Batch or Lot Number</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2146,7 @@
       </c>
       <c r="D59" s="15" t="inlineStr">
         <is>
-          <t>Vaccination notes…</t>
+          <t>Any notes about this vaccination.</t>
         </is>
       </c>
       <c r="E59" s="15" t="n"/>
@@ -2121,7 +2231,12 @@
       </c>
       <c r="K63" s="15" t="inlineStr">
         <is>
-          <t>Only one Mortality event is allowed per animal</t>
+          <t>Only one death (mortality) event can be recorded for each animal.</t>
+        </is>
+      </c>
+      <c r="N63" s="15" t="inlineStr">
+        <is>
+          <t>Select the event type.</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2273,12 @@
       </c>
       <c r="K64" s="15" t="inlineStr">
         <is>
-          <t>Event date must not be in the future</t>
+          <t>The event date cannot be in the future.</t>
+        </is>
+      </c>
+      <c r="N64" s="15" t="inlineStr">
+        <is>
+          <t>Enter the event date.</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2439,12 @@
       </c>
       <c r="K71" s="15" t="inlineStr">
         <is>
-          <t>Number of offspring cannot be negative</t>
+          <t>Enter 0 or more offspring.</t>
+        </is>
+      </c>
+      <c r="N71" s="15" t="inlineStr">
+        <is>
+          <t>Enter the number of offspring.</t>
         </is>
       </c>
     </row>
@@ -2342,6 +2467,11 @@
       <c r="E72" s="15" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="N72" s="15" t="inlineStr">
+        <is>
+          <t>Select the sex of offspring.</t>
         </is>
       </c>
     </row>
@@ -2409,6 +2539,11 @@
           <t>minimal</t>
         </is>
       </c>
+      <c r="N75" s="15" t="inlineStr">
+        <is>
+          <t>Select the disease / diagnosis.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="13.5" customFormat="1" customHeight="1" s="15">
       <c r="A76" s="15" t="inlineStr">
@@ -2433,7 +2568,7 @@
       </c>
       <c r="K76" s="15" t="inlineStr">
         <is>
-          <t>Onset date must not be in the future, and this disease with this onset date is already entered for this animal</t>
+          <t>The onset date cannot be in the future, and the same disease with the same onset date cannot be entered twice for one animal.</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2595,7 @@
       </c>
       <c r="K77" s="15" t="inlineStr">
         <is>
-          <t>Resolution date must be on or after the onset date and not in the future</t>
+          <t>The resolution date must be on or after the onset date and cannot be in the future.</t>
         </is>
       </c>
     </row>
@@ -2480,6 +2615,11 @@
           <t>Notifiable Disease</t>
         </is>
       </c>
+      <c r="D78" s="15" t="inlineStr">
+        <is>
+          <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="13.5" customFormat="1" customHeight="1" s="15">
       <c r="A79" s="15" t="inlineStr">
@@ -2531,7 +2671,11 @@
           <t>Notifiable Disease</t>
         </is>
       </c>
-      <c r="D81" s="15" t="n"/>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
+        </is>
+      </c>
       <c r="E81" s="15" t="n"/>
       <c r="F81" s="15" t="n"/>
       <c r="G81" s="15" t="n"/>
@@ -2663,7 +2807,12 @@
       </c>
       <c r="K87" s="15" t="inlineStr">
         <is>
-          <t>Only female animals can have breeding events</t>
+          <t>Only female animals can have breeding events. Check the sex recorded for this animal.</t>
+        </is>
+      </c>
+      <c r="N87" s="15" t="inlineStr">
+        <is>
+          <t>Select the breeding type.</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2849,12 @@
       </c>
       <c r="K88" s="15" t="inlineStr">
         <is>
-          <t>Breeding date must not be in the future, and this breeding event is already entered for this animal</t>
+          <t>The breeding date cannot be in the future, and the same breeding event with the same date cannot be entered twice for one animal.</t>
+        </is>
+      </c>
+      <c r="N88" s="15" t="inlineStr">
+        <is>
+          <t>Enter the breeding date.</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2971,7 @@
       </c>
       <c r="K94" s="15" t="inlineStr">
         <is>
-          <t>Expected calving date must not be before the breeding date</t>
+          <t>The expected calving date cannot be before the breeding date.</t>
         </is>
       </c>
     </row>
@@ -2866,7 +3020,7 @@
       </c>
       <c r="K96" s="15" t="inlineStr">
         <is>
-          <t>Pregnancy confirmation date must not be in the future</t>
+          <t>The pregnancy confirmation date cannot be in the future.</t>
         </is>
       </c>
     </row>
@@ -2968,12 +3122,17 @@
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
-          <t>AI Technician</t>
+          <t>Artificial Insemination Technician</t>
         </is>
       </c>
       <c r="E100" s="15" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="N100" s="15" t="inlineStr">
+        <is>
+          <t>Enter the name or ID of the artificial insemination technician.</t>
         </is>
       </c>
     </row>
@@ -2990,7 +3149,7 @@
       </c>
       <c r="C101" s="15" t="inlineStr">
         <is>
-          <t>Technique used</t>
+          <t>Technique Used</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4431,7 @@
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Apis Mellifera Scutellata</t>
+          <t>African Honey Bee (Apis mellifera scutellata)</t>
         </is>
       </c>
       <c r="D58" s="15" t="inlineStr">
@@ -4430,7 +4589,7 @@
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Up-to-date</t>
+          <t>Up to date</t>
         </is>
       </c>
     </row>
@@ -5367,7 +5526,7 @@
       </c>
       <c r="C125" s="15" t="inlineStr">
         <is>
-          <t>Marek Disease</t>
+          <t>Marek's Disease</t>
         </is>
       </c>
       <c r="D125" s="15" t="inlineStr">
@@ -5627,7 +5786,7 @@
       </c>
       <c r="C144" s="15" t="inlineStr">
         <is>
-          <t>Gumboro</t>
+          <t>Gumboro (Infectious Bursal Disease)</t>
         </is>
       </c>
     </row>
@@ -6079,7 +6238,7 @@
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Make every ODK form text readable: required messages, plain validation messages and hints (#143)
Field names, choice names, constraints and calculations are unchanged. Form
version v5.
</commit_message>
<xml_diff>
--- a/odk/livestock_registry.xlsx
+++ b/odk/livestock_registry.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M106"/>
+  <dimension ref="A1:N106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.4765625" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26.36" customWidth="1" style="15" min="1" max="1"/>
@@ -498,6 +498,11 @@
           <t>choice_filter</t>
         </is>
       </c>
+      <c r="N1" s="15" t="inlineStr">
+        <is>
+          <t>required_message</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="13.5" customHeight="1" s="18">
       <c r="A2" s="15" t="inlineStr">
@@ -558,7 +563,7 @@
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Optional. Format: FR- followed by 10 digits (e.g. FR-1234567890)</t>
+          <t>Optional. FR- followed by 10 digits, for example FR-1234567890.</t>
         </is>
       </c>
       <c r="J5" s="15" t="inlineStr">
@@ -568,7 +573,7 @@
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
-          <t>farmer_id must be FR- followed by exactly 10 digits</t>
+          <t>The Farmer ID must be FR- followed by exactly 10 digits, for example FR-1234567890.</t>
         </is>
       </c>
     </row>
@@ -585,12 +590,12 @@
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>Fayda FAN ID</t>
+          <t>Fayda FAN (16-digit Fayda number)</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>Format: exactly 16 digits</t>
+          <t>The 16-digit Fayda number, digits only.</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
@@ -607,11 +612,16 @@
       </c>
       <c r="K6" s="21" t="inlineStr">
         <is>
-          <t>Fayda ID must contain exactly 16 digits.</t>
+          <t>Enter the 16-digit Fayda number, using digits only.</t>
         </is>
       </c>
       <c r="L6" s="20" t="n"/>
       <c r="M6" s="20" t="n"/>
+      <c r="N6" s="15" t="inlineStr">
+        <is>
+          <t>Enter the 16-digit Fayda number.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customFormat="1" customHeight="1" s="15">
       <c r="A7" s="20" t="inlineStr">
@@ -641,6 +651,11 @@
       <c r="K7" s="23" t="n"/>
       <c r="L7" s="20" t="n"/>
       <c r="M7" s="20" t="n"/>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>Enter the first name.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customFormat="1" customHeight="1" s="15">
       <c r="A8" s="20" t="inlineStr">
@@ -688,6 +703,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Enter the last name.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="13.5" customHeight="1" s="18">
       <c r="A10" s="15" t="inlineStr">
@@ -729,7 +749,7 @@
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>Date of birth must not be in the future</t>
+          <t>The date of birth cannot be in the future.</t>
         </is>
       </c>
     </row>
@@ -751,7 +771,7 @@
       </c>
       <c r="D12" s="21" t="inlineStr">
         <is>
-          <t>Format: 0911223344 or +251911223344</t>
+          <t>For example 0911223344 or +251911223344.</t>
         </is>
       </c>
       <c r="I12" s="15" t="inlineStr">
@@ -766,7 +786,7 @@
       </c>
       <c r="K12" s="21" t="inlineStr">
         <is>
-          <t>Enter valid Ethiopian number: 0911223344 or +251911223344</t>
+          <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
     </row>
@@ -803,12 +823,17 @@
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>Registration date must not be in the future</t>
+          <t>The registration date cannot be in the future.</t>
         </is>
       </c>
       <c r="L13" s="15" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Enter the registration date.</t>
         </is>
       </c>
     </row>
@@ -862,7 +887,7 @@
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>DA Name</t>
+          <t>Development Agent Name</t>
         </is>
       </c>
       <c r="D16" s="20" t="n"/>
@@ -888,12 +913,12 @@
       </c>
       <c r="C17" s="20" t="inlineStr">
         <is>
-          <t>DA Mobile Number</t>
+          <t>Development Agent Mobile Number</t>
         </is>
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
-          <t>Format: 0911223344 or +251911223344</t>
+          <t>For example 0911223344 or +251911223344.</t>
         </is>
       </c>
       <c r="E17" s="20" t="n"/>
@@ -910,7 +935,7 @@
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
-          <t>Enter valid Ethiopian number: 0911223344 or +251911223344</t>
+          <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
       <c r="L17" s="20" t="n"/>
@@ -959,7 +984,7 @@
       </c>
       <c r="D19" s="21" t="inlineStr">
         <is>
-          <t>Format: 0911223344 or +251911223344</t>
+          <t>For example 0911223344 or +251911223344.</t>
         </is>
       </c>
       <c r="E19" s="20" t="n"/>
@@ -976,7 +1001,7 @@
       </c>
       <c r="K19" s="21" t="inlineStr">
         <is>
-          <t>Enter valid Ethiopian number: 0911223344 or +251911223344</t>
+          <t>Enter a valid Ethiopian mobile number, for example 0911223344 or +251911223344.</t>
         </is>
       </c>
       <c r="L19" s="20" t="n"/>
@@ -1182,6 +1207,11 @@
         </is>
       </c>
       <c r="J28" s="21" t="n"/>
+      <c r="N28" s="15" t="inlineStr">
+        <is>
+          <t>Select the species.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1" s="18">
       <c r="A29" s="15" t="inlineStr">
@@ -1216,6 +1246,11 @@
           <t>species = ${species_id}</t>
         </is>
       </c>
+      <c r="N29" s="15" t="inlineStr">
+        <is>
+          <t>Select the breed.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="18">
       <c r="A30" s="15" t="inlineStr">
@@ -1235,7 +1270,7 @@
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>Ear tag ID must be in format ET0000000000</t>
+          <t>ET followed by 10 digits, for example ET0123456789.</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
@@ -1255,7 +1290,12 @@
       </c>
       <c r="K30" s="15" t="inlineStr">
         <is>
-          <t>Ear tag must be ET + 10 digits (e.g. ET0000000000) and must not be repeated in this record</t>
+          <t>Enter the ear tag as ET followed by 10 digits, for example ET0123456789. Each animal in this record needs a different ear tag.</t>
+        </is>
+      </c>
+      <c r="N30" s="15" t="inlineStr">
+        <is>
+          <t>Enter the livestock ear tag.</t>
         </is>
       </c>
     </row>
@@ -1292,10 +1332,15 @@
       </c>
       <c r="K31" s="15" t="inlineStr">
         <is>
-          <t>This secondary identifier is used more than once in this record</t>
+          <t>This identifier is already used by another animal in this record. Enter a different one.</t>
         </is>
       </c>
       <c r="M31" s="21" t="n"/>
+      <c r="N31" s="15" t="inlineStr">
+        <is>
+          <t>Enter the secondary identifier (leg band / wing tag / hive number).</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="30" customHeight="1" s="18">
       <c r="A32" s="15" t="inlineStr">
@@ -1310,7 +1355,7 @@
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Quantity (Head Count)</t>
+          <t>Number of Animals or Hives</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
@@ -1330,10 +1375,15 @@
       </c>
       <c r="K32" s="15" t="inlineStr">
         <is>
-          <t>Quantity must be greater than 0</t>
+          <t>Enter a number greater than 0.</t>
         </is>
       </c>
       <c r="M32" s="21" t="n"/>
+      <c r="N32" s="15" t="inlineStr">
+        <is>
+          <t>Enter the number of animals or hives.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="13.5" customHeight="1" s="18">
       <c r="A33" s="15" t="inlineStr">
@@ -1358,7 +1408,7 @@
       </c>
       <c r="K33" s="15" t="inlineStr">
         <is>
-          <t>Weight must be greater than 0</t>
+          <t>Enter a weight greater than 0 kg.</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1445,12 @@
       </c>
       <c r="K34" s="15" t="inlineStr">
         <is>
-          <t>Date of birth must not be in the future</t>
+          <t>The date of birth cannot be in the future.</t>
+        </is>
+      </c>
+      <c r="N34" s="15" t="inlineStr">
+        <is>
+          <t>Enter the date of birth.</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1482,12 @@
       </c>
       <c r="K35" s="15" t="inlineStr">
         <is>
-          <t>'Mixed / Not Applicable' is allowed only for poultry and beehive</t>
+          <t>Mixed / Not Applicable can only be chosen for poultry and beehives. Choose Male or Female.</t>
+        </is>
+      </c>
+      <c r="N35" s="15" t="inlineStr">
+        <is>
+          <t>Select the sex.</t>
         </is>
       </c>
     </row>
@@ -1462,6 +1522,11 @@
           <t>minimal</t>
         </is>
       </c>
+      <c r="N36" s="15" t="inlineStr">
+        <is>
+          <t>Select the health status.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="13.5" customHeight="1" s="18">
       <c r="A37" s="15" t="inlineStr">
@@ -1494,6 +1559,11 @@
           <t>minimal</t>
         </is>
       </c>
+      <c r="N37" s="15" t="inlineStr">
+        <is>
+          <t>Select the vaccination status.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="13.5" customHeight="1" s="18">
       <c r="A38" s="15" t="inlineStr">
@@ -1528,12 +1598,17 @@
       </c>
       <c r="K38" s="15" t="inlineStr">
         <is>
-          <t>Registration date must not be in the future</t>
+          <t>The registration date cannot be in the future.</t>
         </is>
       </c>
       <c r="L38" s="15" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="N38" s="15" t="inlineStr">
+        <is>
+          <t>Enter the registration date.</t>
         </is>
       </c>
     </row>
@@ -1591,6 +1666,11 @@
           <t>minimal</t>
         </is>
       </c>
+      <c r="N41" s="15" t="inlineStr">
+        <is>
+          <t>Select the event type.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="18">
       <c r="A42" s="15" t="inlineStr">
@@ -1623,6 +1703,11 @@
           <t>minimal</t>
         </is>
       </c>
+      <c r="N42" s="15" t="inlineStr">
+        <is>
+          <t>Select the disease.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1" s="18">
       <c r="A43" s="15" t="inlineStr">
@@ -1657,7 +1742,12 @@
       </c>
       <c r="K43" s="15" t="inlineStr">
         <is>
-          <t>Onset date must not be in the future, and this event (same type and onset date) is already entered for this animal</t>
+          <t>The onset date cannot be in the future, and the same event with the same onset date cannot be entered twice for one animal.</t>
+        </is>
+      </c>
+      <c r="N43" s="15" t="inlineStr">
+        <is>
+          <t>Enter the date of onset.</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1784,12 @@
       </c>
       <c r="K44" s="15" t="inlineStr">
         <is>
-          <t>Resolution date must be on or after the onset date and not in the future</t>
+          <t>The resolution date must be on or after the onset date and cannot be in the future.</t>
+        </is>
+      </c>
+      <c r="N44" s="15" t="inlineStr">
+        <is>
+          <t>Enter the date of resolution.</t>
         </is>
       </c>
     </row>
@@ -1714,6 +1809,11 @@
           <t>Notifiable Disease</t>
         </is>
       </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
+        </is>
+      </c>
       <c r="F45" s="15" t="inlineStr">
         <is>
           <t>no</t>
@@ -1814,7 +1914,7 @@
       </c>
       <c r="D49" s="15" t="inlineStr">
         <is>
-          <t>e.g. exact address, clinic name</t>
+          <t>For example the exact address or the clinic name.</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1936,7 @@
       </c>
       <c r="D50" s="15" t="inlineStr">
         <is>
-          <t>Additional notes…</t>
+          <t>Any additional notes.</t>
         </is>
       </c>
       <c r="E50" s="15" t="n"/>
@@ -1919,6 +2019,11 @@
           <t>species = ${species_id}</t>
         </is>
       </c>
+      <c r="N54" s="15" t="inlineStr">
+        <is>
+          <t>Select the vaccine.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="13.5" customHeight="1" s="18">
       <c r="A55" s="15" t="inlineStr">
@@ -1953,7 +2058,12 @@
       </c>
       <c r="K55" s="15" t="inlineStr">
         <is>
-          <t>Vaccination date must not be in the future, and this vaccine on this date is already entered for this animal</t>
+          <t>The vaccination date cannot be in the future, and the same vaccine with the same date cannot be entered twice for one animal.</t>
+        </is>
+      </c>
+      <c r="N55" s="15" t="inlineStr">
+        <is>
+          <t>Enter the vaccination date.</t>
         </is>
       </c>
     </row>
@@ -1980,7 +2090,7 @@
       </c>
       <c r="K56" s="15" t="inlineStr">
         <is>
-          <t>Next due date must not be before the vaccination date</t>
+          <t>The next due date cannot be before the vaccination date.</t>
         </is>
       </c>
     </row>
@@ -1997,7 +2107,7 @@
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>Batch/Lot Number</t>
+          <t>Batch or Lot Number</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2146,7 @@
       </c>
       <c r="D59" s="15" t="inlineStr">
         <is>
-          <t>Vaccination notes…</t>
+          <t>Any notes about this vaccination.</t>
         </is>
       </c>
       <c r="E59" s="15" t="n"/>
@@ -2121,7 +2231,12 @@
       </c>
       <c r="K63" s="15" t="inlineStr">
         <is>
-          <t>Only one Mortality event is allowed per animal</t>
+          <t>Only one death (mortality) event can be recorded for each animal.</t>
+        </is>
+      </c>
+      <c r="N63" s="15" t="inlineStr">
+        <is>
+          <t>Select the event type.</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2273,12 @@
       </c>
       <c r="K64" s="15" t="inlineStr">
         <is>
-          <t>Event date must not be in the future</t>
+          <t>The event date cannot be in the future.</t>
+        </is>
+      </c>
+      <c r="N64" s="15" t="inlineStr">
+        <is>
+          <t>Enter the event date.</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2439,12 @@
       </c>
       <c r="K71" s="15" t="inlineStr">
         <is>
-          <t>Number of offspring cannot be negative</t>
+          <t>Enter 0 or more offspring.</t>
+        </is>
+      </c>
+      <c r="N71" s="15" t="inlineStr">
+        <is>
+          <t>Enter the number of offspring.</t>
         </is>
       </c>
     </row>
@@ -2342,6 +2467,11 @@
       <c r="E72" s="15" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="N72" s="15" t="inlineStr">
+        <is>
+          <t>Select the sex of offspring.</t>
         </is>
       </c>
     </row>
@@ -2409,6 +2539,11 @@
           <t>minimal</t>
         </is>
       </c>
+      <c r="N75" s="15" t="inlineStr">
+        <is>
+          <t>Select the disease / diagnosis.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="13.5" customFormat="1" customHeight="1" s="15">
       <c r="A76" s="15" t="inlineStr">
@@ -2433,7 +2568,7 @@
       </c>
       <c r="K76" s="15" t="inlineStr">
         <is>
-          <t>Onset date must not be in the future, and this disease with this onset date is already entered for this animal</t>
+          <t>The onset date cannot be in the future, and the same disease with the same onset date cannot be entered twice for one animal.</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2595,7 @@
       </c>
       <c r="K77" s="15" t="inlineStr">
         <is>
-          <t>Resolution date must be on or after the onset date and not in the future</t>
+          <t>The resolution date must be on or after the onset date and cannot be in the future.</t>
         </is>
       </c>
     </row>
@@ -2480,6 +2615,11 @@
           <t>Notifiable Disease</t>
         </is>
       </c>
+      <c r="D78" s="15" t="inlineStr">
+        <is>
+          <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="13.5" customFormat="1" customHeight="1" s="15">
       <c r="A79" s="15" t="inlineStr">
@@ -2531,7 +2671,11 @@
           <t>Notifiable Disease</t>
         </is>
       </c>
-      <c r="D81" s="15" t="n"/>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
+        </is>
+      </c>
       <c r="E81" s="15" t="n"/>
       <c r="F81" s="15" t="n"/>
       <c r="G81" s="15" t="n"/>
@@ -2663,7 +2807,12 @@
       </c>
       <c r="K87" s="15" t="inlineStr">
         <is>
-          <t>Only female animals can have breeding events</t>
+          <t>Only female animals can have breeding events. Check the sex recorded for this animal.</t>
+        </is>
+      </c>
+      <c r="N87" s="15" t="inlineStr">
+        <is>
+          <t>Select the breeding type.</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2849,12 @@
       </c>
       <c r="K88" s="15" t="inlineStr">
         <is>
-          <t>Breeding date must not be in the future, and this breeding event is already entered for this animal</t>
+          <t>The breeding date cannot be in the future, and the same breeding event with the same date cannot be entered twice for one animal.</t>
+        </is>
+      </c>
+      <c r="N88" s="15" t="inlineStr">
+        <is>
+          <t>Enter the breeding date.</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2971,7 @@
       </c>
       <c r="K94" s="15" t="inlineStr">
         <is>
-          <t>Expected calving date must not be before the breeding date</t>
+          <t>The expected calving date cannot be before the breeding date.</t>
         </is>
       </c>
     </row>
@@ -2866,7 +3020,7 @@
       </c>
       <c r="K96" s="15" t="inlineStr">
         <is>
-          <t>Pregnancy confirmation date must not be in the future</t>
+          <t>The pregnancy confirmation date cannot be in the future.</t>
         </is>
       </c>
     </row>
@@ -2968,12 +3122,17 @@
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
-          <t>AI Technician</t>
+          <t>Artificial Insemination Technician</t>
         </is>
       </c>
       <c r="E100" s="15" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="N100" s="15" t="inlineStr">
+        <is>
+          <t>Enter the name or ID of the artificial insemination technician.</t>
         </is>
       </c>
     </row>
@@ -2990,7 +3149,7 @@
       </c>
       <c r="C101" s="15" t="inlineStr">
         <is>
-          <t>Technique used</t>
+          <t>Technique Used</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4431,7 @@
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Apis Mellifera Scutellata</t>
+          <t>African Honey Bee (Apis mellifera scutellata)</t>
         </is>
       </c>
       <c r="D58" s="15" t="inlineStr">
@@ -4430,7 +4589,7 @@
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Up-to-date</t>
+          <t>Up to date</t>
         </is>
       </c>
     </row>
@@ -5367,7 +5526,7 @@
       </c>
       <c r="C125" s="15" t="inlineStr">
         <is>
-          <t>Marek Disease</t>
+          <t>Marek's Disease</t>
         </is>
       </c>
       <c r="D125" s="15" t="inlineStr">
@@ -5627,7 +5786,7 @@
       </c>
       <c r="C144" s="15" t="inlineStr">
         <is>
-          <t>Gumboro</t>
+          <t>Gumboro (Infectious Bursal Disease)</t>
         </is>
       </c>
     </row>
@@ -6079,7 +6238,7 @@
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Livestock ODK form: Farmer ID is FR- and 12 digits, Fayda ID is a 16-digit FAN or a 12-digit FIN
Matches the registry and the Farmer and Crop forms. The transform already maps a
12-digit value to the FIN and any other value to the FAN. Form version v6.
</commit_message>
<xml_diff>
--- a/odk/livestock_registry.xlsx
+++ b/odk/livestock_registry.xlsx
@@ -563,17 +563,17 @@
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Optional. FR- followed by 10 digits, for example FR-1234567890.</t>
+          <t>Optional. FR- followed by 12 digits, for example FR-123456789012.</t>
         </is>
       </c>
       <c r="J5" s="15" t="inlineStr">
         <is>
-          <t>regex(., '^FR-[0-9]{10}$')</t>
+          <t>regex(., '^FR-[0-9]{12}$')</t>
         </is>
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
-          <t>The Farmer ID must be FR- followed by exactly 10 digits, for example FR-1234567890.</t>
+          <t>The Farmer ID must be FR- followed by 12 digits, for example FR-123456789012.</t>
         </is>
       </c>
     </row>
@@ -590,12 +590,12 @@
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>Fayda FAN (16-digit Fayda number)</t>
+          <t>Fayda ID</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>The 16-digit Fayda number, digits only.</t>
+          <t>The 16-digit FAN or the 12-digit FIN, digits only.</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
@@ -607,19 +607,19 @@
       <c r="I6" s="20" t="n"/>
       <c r="J6" s="21" t="inlineStr">
         <is>
-          <t>regex(., '^[0-9]{16}$')</t>
+          <t>regex(., '^([0-9]{12}|[0-9]{16})$')</t>
         </is>
       </c>
       <c r="K6" s="21" t="inlineStr">
         <is>
-          <t>Enter the 16-digit Fayda number, using digits only.</t>
+          <t>The Fayda ID must be a 16-digit FAN or a 12-digit FIN, using digits only.</t>
         </is>
       </c>
       <c r="L6" s="20" t="n"/>
       <c r="M6" s="20" t="n"/>
       <c r="N6" s="15" t="inlineStr">
         <is>
-          <t>Enter the 16-digit Fayda number.</t>
+          <t>Enter the Fayda ID.</t>
         </is>
       </c>
     </row>
@@ -6238,7 +6238,7 @@
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>v5</t>
+          <t>v6</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Livestock ODK form: Farmer ID is FR- and 12 digits, Fayda ID is a 16-digit FAN or a 12-digit FIN (#146)
Matches the registry and the Farmer and Crop forms. The transform already maps a
12-digit value to the FIN and any other value to the FAN. Form version v6.
</commit_message>
<xml_diff>
--- a/odk/livestock_registry.xlsx
+++ b/odk/livestock_registry.xlsx
@@ -563,17 +563,17 @@
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Optional. FR- followed by 10 digits, for example FR-1234567890.</t>
+          <t>Optional. FR- followed by 12 digits, for example FR-123456789012.</t>
         </is>
       </c>
       <c r="J5" s="15" t="inlineStr">
         <is>
-          <t>regex(., '^FR-[0-9]{10}$')</t>
+          <t>regex(., '^FR-[0-9]{12}$')</t>
         </is>
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
-          <t>The Farmer ID must be FR- followed by exactly 10 digits, for example FR-1234567890.</t>
+          <t>The Farmer ID must be FR- followed by 12 digits, for example FR-123456789012.</t>
         </is>
       </c>
     </row>
@@ -590,12 +590,12 @@
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>Fayda FAN (16-digit Fayda number)</t>
+          <t>Fayda ID</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>The 16-digit Fayda number, digits only.</t>
+          <t>The 16-digit FAN or the 12-digit FIN, digits only.</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
@@ -607,19 +607,19 @@
       <c r="I6" s="20" t="n"/>
       <c r="J6" s="21" t="inlineStr">
         <is>
-          <t>regex(., '^[0-9]{16}$')</t>
+          <t>regex(., '^([0-9]{12}|[0-9]{16})$')</t>
         </is>
       </c>
       <c r="K6" s="21" t="inlineStr">
         <is>
-          <t>Enter the 16-digit Fayda number, using digits only.</t>
+          <t>The Fayda ID must be a 16-digit FAN or a 12-digit FIN, using digits only.</t>
         </is>
       </c>
       <c r="L6" s="20" t="n"/>
       <c r="M6" s="20" t="n"/>
       <c r="N6" s="15" t="inlineStr">
         <is>
-          <t>Enter the 16-digit Fayda number.</t>
+          <t>Enter the Fayda ID.</t>
         </is>
       </c>
     </row>
@@ -6238,7 +6238,7 @@
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>v5</t>
+          <t>v6</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Livestock ODK form v7: pick locations by Master Data codes
The form sent old names and codes, so the transform never saw
location_source=mds and ingestion stopped on the empty administrative
hierarchy. The location questions are now region_code ... kebele_code with a
hidden location_source=mds, and the four choice lists are generated from the
ETH-OAN pack (names are the Master Data ids, labels are readable names).
Adds the generator, v7-shaped samples and a transform test.
</commit_message>
<xml_diff>
--- a/odk/livestock_registry.xlsx
+++ b/odk/livestock_registry.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N106"/>
+  <dimension ref="A1:N107"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.4765625" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26.36" customWidth="1" style="15" min="1" max="1"/>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>region_id</t>
+          <t>region_code</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>zone_id</t>
+          <t>zone_code</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="M23" s="21" t="inlineStr">
         <is>
-          <t>region=${region_id}</t>
+          <t>region=${region_code}</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>woreda_id</t>
+          <t>woreda_code</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="M24" s="21" t="inlineStr">
         <is>
-          <t>zone=${zone_id}</t>
+          <t>zone=${zone_code}</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>kebele_id</t>
+          <t>kebele_code</t>
         </is>
       </c>
       <c r="C25" s="15" t="inlineStr">
@@ -1141,92 +1141,75 @@
       </c>
       <c r="M25" s="15" t="inlineStr">
         <is>
-          <t>woreda=${woreda_id}</t>
+          <t>woreda=${woreda_code}</t>
         </is>
       </c>
     </row>
     <row r="26" ht="13.5" customFormat="1" customHeight="1" s="19">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>end_group</t>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>location_source</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>'mds'</t>
         </is>
       </c>
     </row>
     <row r="27" ht="13.5" customHeight="1" s="18">
       <c r="A27" s="19" t="inlineStr">
         <is>
+          <t>end_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1" s="18">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
           <t>begin_repeat</t>
         </is>
       </c>
-      <c r="B27" s="19" t="inlineStr">
+      <c r="B28" s="19" t="inlineStr">
         <is>
           <t>livestock</t>
         </is>
       </c>
-      <c r="C27" s="19" t="inlineStr">
+      <c r="C28" s="19" t="inlineStr">
         <is>
           <t>Livestock Animals</t>
         </is>
       </c>
-      <c r="D27" s="19" t="n"/>
-      <c r="E27" s="19" t="n"/>
-      <c r="F27" s="19" t="n"/>
-      <c r="G27" s="19" t="n"/>
-      <c r="H27" s="19" t="n"/>
-      <c r="I27" s="19" t="n"/>
-      <c r="J27" s="19" t="n"/>
-      <c r="K27" s="19" t="n"/>
-      <c r="L27" s="19" t="n"/>
-      <c r="M27" s="19" t="n"/>
-    </row>
-    <row r="28" ht="30" customHeight="1" s="18">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>select_one species</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>species_id</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="E28" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G28" s="21" t="n"/>
-      <c r="I28" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="J28" s="21" t="n"/>
-      <c r="N28" s="15" t="inlineStr">
-        <is>
-          <t>Select the species.</t>
-        </is>
-      </c>
+      <c r="D28" s="19" t="n"/>
+      <c r="E28" s="19" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="19" t="n"/>
+      <c r="H28" s="19" t="n"/>
+      <c r="I28" s="19" t="n"/>
+      <c r="J28" s="19" t="n"/>
+      <c r="K28" s="19" t="n"/>
+      <c r="L28" s="19" t="n"/>
+      <c r="M28" s="19" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1" s="18">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>select_one breed</t>
+          <t>select_one species</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>breed</t>
+          <t>species_id</t>
         </is>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>Breed</t>
+          <t>Species</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
@@ -1241,36 +1224,26 @@
         </is>
       </c>
       <c r="J29" s="21" t="n"/>
-      <c r="M29" s="15" t="inlineStr">
-        <is>
-          <t>species = ${species_id}</t>
-        </is>
-      </c>
       <c r="N29" s="15" t="inlineStr">
         <is>
-          <t>Select the breed.</t>
+          <t>Select the species.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="18">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one breed</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>ear_tag_id</t>
+          <t>breed</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>Livestock Ear Tag</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="inlineStr">
-        <is>
-          <t>ET followed by 10 digits, for example ET0123456789.</t>
+          <t>Breed</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
@@ -1278,24 +1251,21 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G30" s="15" t="inlineStr">
-        <is>
-          <t>not(selected(${species_id}, 'poultry')) and not(selected(${species_id}, 'beehive'))</t>
-        </is>
-      </c>
-      <c r="J30" s="15" t="inlineStr">
-        <is>
-          <t>regex(., '^ET[0-9]{10}$') and not(contains(substring-after(join(' ', ../../livestock/ear_tag_id), .), .))</t>
-        </is>
-      </c>
-      <c r="K30" s="15" t="inlineStr">
-        <is>
-          <t>Enter the ear tag as ET followed by 10 digits, for example ET0123456789. Each animal in this record needs a different ear tag.</t>
+      <c r="G30" s="21" t="n"/>
+      <c r="I30" s="15" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="J30" s="21" t="n"/>
+      <c r="M30" s="15" t="inlineStr">
+        <is>
+          <t>species = ${species_id}</t>
         </is>
       </c>
       <c r="N30" s="15" t="inlineStr">
         <is>
-          <t>Enter the livestock ear tag.</t>
+          <t>Select the breed.</t>
         </is>
       </c>
     </row>
@@ -1307,12 +1277,17 @@
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>secondary_identifier</t>
+          <t>ear_tag_id</t>
         </is>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>Secondary Identifier (leg band / wing tag / hive number)</t>
+          <t>Livestock Ear Tag</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>ET followed by 10 digits, for example ET0123456789.</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
@@ -1322,40 +1297,39 @@
       </c>
       <c r="G31" s="15" t="inlineStr">
         <is>
-          <t>selected(${species_id}, 'poultry') or selected(${species_id}, 'beehive')</t>
+          <t>not(selected(${species_id}, 'poultry')) and not(selected(${species_id}, 'beehive'))</t>
         </is>
       </c>
       <c r="J31" s="15" t="inlineStr">
         <is>
-          <t>not(contains(concat('|', substring-after(concat('|', join('|', ../../livestock/secondary_identifier), '|'), concat('|', ., '|'))), concat('|', ., '|')))</t>
+          <t>regex(., '^ET[0-9]{10}$') and not(contains(substring-after(join(' ', ../../livestock/ear_tag_id), .), .))</t>
         </is>
       </c>
       <c r="K31" s="15" t="inlineStr">
         <is>
-          <t>This identifier is already used by another animal in this record. Enter a different one.</t>
-        </is>
-      </c>
-      <c r="M31" s="21" t="n"/>
+          <t>Enter the ear tag as ET followed by 10 digits, for example ET0123456789. Each animal in this record needs a different ear tag.</t>
+        </is>
+      </c>
       <c r="N31" s="15" t="inlineStr">
         <is>
-          <t>Enter the secondary identifier (leg band / wing tag / hive number).</t>
+          <t>Enter the livestock ear tag.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" s="18">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>secondary_identifier</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Number of Animals or Hives</t>
+          <t>Secondary Identifier (leg band / wing tag / hive number)</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
@@ -1363,42 +1337,52 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G32" s="21" t="inlineStr">
+      <c r="G32" s="15" t="inlineStr">
         <is>
           <t>selected(${species_id}, 'poultry') or selected(${species_id}, 'beehive')</t>
         </is>
       </c>
       <c r="J32" s="15" t="inlineStr">
         <is>
-          <t>. &gt; 0</t>
+          <t>not(contains(concat('|', substring-after(concat('|', join('|', ../../livestock/secondary_identifier), '|'), concat('|', ., '|'))), concat('|', ., '|')))</t>
         </is>
       </c>
       <c r="K32" s="15" t="inlineStr">
         <is>
-          <t>Enter a number greater than 0.</t>
+          <t>This identifier is already used by another animal in this record. Enter a different one.</t>
         </is>
       </c>
       <c r="M32" s="21" t="n"/>
       <c r="N32" s="15" t="inlineStr">
         <is>
-          <t>Enter the number of animals or hives.</t>
+          <t>Enter the secondary identifier (leg band / wing tag / hive number).</t>
         </is>
       </c>
     </row>
     <row r="33" ht="13.5" customHeight="1" s="18">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Weight (kg)</t>
+          <t>Number of Animals or Hives</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G33" s="21" t="inlineStr">
+        <is>
+          <t>selected(${species_id}, 'poultry') or selected(${species_id}, 'beehive')</t>
         </is>
       </c>
       <c r="J33" s="15" t="inlineStr">
@@ -1408,66 +1392,57 @@
       </c>
       <c r="K33" s="15" t="inlineStr">
         <is>
-          <t>Enter a weight greater than 0 kg.</t>
+          <t>Enter a number greater than 0.</t>
+        </is>
+      </c>
+      <c r="M33" s="21" t="n"/>
+      <c r="N33" s="15" t="inlineStr">
+        <is>
+          <t>Enter the number of animals or hives.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="13.5" customHeight="1" s="18">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>date_of_birth</t>
+          <t>weight</t>
         </is>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>Date of Birth</t>
-        </is>
-      </c>
-      <c r="E34" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G34" s="15" t="inlineStr">
-        <is>
-          <t>not(selected(${species_id}, 'poultry')) and not(selected(${species_id}, 'beehive'))</t>
+          <t>Weight (kg)</t>
         </is>
       </c>
       <c r="J34" s="15" t="inlineStr">
         <is>
-          <t>. &lt;= today()</t>
+          <t>. &gt; 0</t>
         </is>
       </c>
       <c r="K34" s="15" t="inlineStr">
         <is>
-          <t>The date of birth cannot be in the future.</t>
-        </is>
-      </c>
-      <c r="N34" s="15" t="inlineStr">
-        <is>
-          <t>Enter the date of birth.</t>
+          <t>Enter a weight greater than 0 kg.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="13.5" customHeight="1" s="18">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>select_one animal_sex</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>date_of_birth</t>
         </is>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Date of Birth</t>
         </is>
       </c>
       <c r="E35" s="15" t="inlineStr">
@@ -1475,36 +1450,41 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>not(selected(${species_id}, 'poultry')) and not(selected(${species_id}, 'beehive'))</t>
+        </is>
+      </c>
       <c r="J35" s="15" t="inlineStr">
         <is>
-          <t>not(. = 'mixed') or (selected(${species_id}, 'poultry') or selected(${species_id}, 'beehive'))</t>
+          <t>. &lt;= today()</t>
         </is>
       </c>
       <c r="K35" s="15" t="inlineStr">
         <is>
-          <t>Mixed / Not Applicable can only be chosen for poultry and beehives. Choose Male or Female.</t>
+          <t>The date of birth cannot be in the future.</t>
         </is>
       </c>
       <c r="N35" s="15" t="inlineStr">
         <is>
-          <t>Select the sex.</t>
+          <t>Enter the date of birth.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="13.5" customHeight="1" s="18">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>select_one health_status</t>
+          <t>select_one animal_sex</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>health_status</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>Health Status</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="E36" s="15" t="inlineStr">
@@ -1512,36 +1492,36 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F36" s="15" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="I36" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
+      <c r="J36" s="15" t="inlineStr">
+        <is>
+          <t>not(. = 'mixed') or (selected(${species_id}, 'poultry') or selected(${species_id}, 'beehive'))</t>
+        </is>
+      </c>
+      <c r="K36" s="15" t="inlineStr">
+        <is>
+          <t>Mixed / Not Applicable can only be chosen for poultry and beehives. Choose Male or Female.</t>
         </is>
       </c>
       <c r="N36" s="15" t="inlineStr">
         <is>
-          <t>Select the health status.</t>
+          <t>Select the sex.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="13.5" customHeight="1" s="18">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>select_one vaccination_status</t>
+          <t>select_one health_status</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>vaccination_status</t>
+          <t>health_status</t>
         </is>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Vaccination Status</t>
+          <t>Health Status</t>
         </is>
       </c>
       <c r="E37" s="15" t="inlineStr">
@@ -1551,7 +1531,7 @@
       </c>
       <c r="F37" s="15" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="I37" s="15" t="inlineStr">
@@ -1561,131 +1541,136 @@
       </c>
       <c r="N37" s="15" t="inlineStr">
         <is>
-          <t>Select the vaccination status.</t>
+          <t>Select the health status.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="13.5" customHeight="1" s="18">
       <c r="A38" s="15" t="inlineStr">
         <is>
+          <t>select_one vaccination_status</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>vaccination_status</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>Vaccination Status</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F38" s="15" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I38" s="15" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="N38" s="15" t="inlineStr">
+        <is>
+          <t>Select the vaccination status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="13.5" customHeight="1" s="18">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B38" s="15" t="inlineStr">
+      <c r="B39" s="15" t="inlineStr">
         <is>
           <t>registration_date</t>
         </is>
       </c>
-      <c r="C38" s="15" t="inlineStr">
+      <c r="C39" s="15" t="inlineStr">
         <is>
           <t>Registration Date</t>
         </is>
       </c>
-      <c r="E38" s="15" t="inlineStr">
+      <c r="E39" s="15" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F38" s="15" t="inlineStr">
+      <c r="F39" s="15" t="inlineStr">
         <is>
           <t>today()</t>
         </is>
       </c>
-      <c r="J38" s="15" t="inlineStr">
+      <c r="J39" s="15" t="inlineStr">
         <is>
           <t>. &lt;= today()</t>
         </is>
       </c>
-      <c r="K38" s="15" t="inlineStr">
+      <c r="K39" s="15" t="inlineStr">
         <is>
           <t>The registration date cannot be in the future.</t>
         </is>
       </c>
-      <c r="L38" s="15" t="inlineStr">
+      <c r="L39" s="15" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="N38" s="15" t="inlineStr">
+      <c r="N39" s="15" t="inlineStr">
         <is>
           <t>Enter the registration date.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="13.5" customHeight="1" s="18"/>
-    <row r="40" ht="13.5" customHeight="1" s="18">
-      <c r="A40" s="19" t="inlineStr">
+    <row r="40" ht="13.5" customHeight="1" s="18"/>
+    <row r="41" ht="13.5" customHeight="1" s="18">
+      <c r="A41" s="19" t="inlineStr">
         <is>
           <t>begin_repeat</t>
         </is>
       </c>
-      <c r="B40" s="19" t="inlineStr">
+      <c r="B41" s="19" t="inlineStr">
         <is>
           <t>health_events</t>
         </is>
       </c>
-      <c r="C40" s="19" t="inlineStr">
+      <c r="C41" s="19" t="inlineStr">
         <is>
           <t>Health Events</t>
         </is>
       </c>
-      <c r="D40" s="19" t="n"/>
-      <c r="E40" s="19" t="n"/>
-      <c r="F40" s="19" t="n"/>
-      <c r="G40" s="19" t="n"/>
-      <c r="H40" s="19" t="n"/>
-      <c r="I40" s="19" t="n"/>
-      <c r="J40" s="19" t="n"/>
-      <c r="K40" s="19" t="n"/>
-      <c r="L40" s="19" t="n"/>
-      <c r="M40" s="19" t="n"/>
-    </row>
-    <row r="41" ht="13.5" customHeight="1" s="18">
-      <c r="A41" s="15" t="inlineStr">
-        <is>
-          <t>select_one health_event_type</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="inlineStr">
-        <is>
-          <t>event_type</t>
-        </is>
-      </c>
-      <c r="C41" s="15" t="inlineStr">
-        <is>
-          <t>Event Type</t>
-        </is>
-      </c>
-      <c r="E41" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I41" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="N41" s="15" t="inlineStr">
-        <is>
-          <t>Select the event type.</t>
-        </is>
-      </c>
+      <c r="D41" s="19" t="n"/>
+      <c r="E41" s="19" t="n"/>
+      <c r="F41" s="19" t="n"/>
+      <c r="G41" s="19" t="n"/>
+      <c r="H41" s="19" t="n"/>
+      <c r="I41" s="19" t="n"/>
+      <c r="J41" s="19" t="n"/>
+      <c r="K41" s="19" t="n"/>
+      <c r="L41" s="19" t="n"/>
+      <c r="M41" s="19" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="18">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>select_one disease</t>
+          <t>select_one health_event_type</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>disease_type</t>
+          <t>event_type</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>Disease</t>
+          <t>Event Type</t>
         </is>
       </c>
       <c r="E42" s="15" t="inlineStr">
@@ -1693,11 +1678,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G42" s="21" t="inlineStr">
-        <is>
-          <t>${event_type} = 'disease'</t>
-        </is>
-      </c>
       <c r="I42" s="15" t="inlineStr">
         <is>
           <t>minimal</t>
@@ -1705,24 +1685,24 @@
       </c>
       <c r="N42" s="15" t="inlineStr">
         <is>
-          <t>Select the disease.</t>
+          <t>Select the event type.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1" s="18">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one disease</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>date_onset</t>
+          <t>disease_type</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>Date of Onset</t>
+          <t>Disease</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
@@ -1732,22 +1712,17 @@
       </c>
       <c r="G43" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">${event_type} = 'disease' or ${event_type} = 'injury' or ${event_type} = 'treatment' </t>
-        </is>
-      </c>
-      <c r="J43" s="15" t="inlineStr">
-        <is>
-          <t>. &lt;= today()</t>
-        </is>
-      </c>
-      <c r="K43" s="15" t="inlineStr">
-        <is>
-          <t>The onset date cannot be in the future, and the same event with the same onset date cannot be entered twice for one animal.</t>
+          <t>${event_type} = 'disease'</t>
+        </is>
+      </c>
+      <c r="I43" s="15" t="inlineStr">
+        <is>
+          <t>minimal</t>
         </is>
       </c>
       <c r="N43" s="15" t="inlineStr">
         <is>
-          <t>Enter the date of onset.</t>
+          <t>Select the disease.</t>
         </is>
       </c>
     </row>
@@ -1759,12 +1734,12 @@
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>date_resolution</t>
+          <t>date_onset</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>Date of Resolution</t>
+          <t>Date of Onset</t>
         </is>
       </c>
       <c r="E44" s="15" t="inlineStr">
@@ -1774,86 +1749,101 @@
       </c>
       <c r="G44" s="21" t="inlineStr">
         <is>
-          <t>${event_type} = 'disease' or ${event_type} = 'injury' or ${event_type} = 'recovery'</t>
+          <t xml:space="preserve">${event_type} = 'disease' or ${event_type} = 'injury' or ${event_type} = 'treatment' </t>
         </is>
       </c>
       <c r="J44" s="15" t="inlineStr">
         <is>
-          <t>(. &gt;= ${date_onset} or ${date_onset} = '') and . &lt;= today()</t>
+          <t>. &lt;= today()</t>
         </is>
       </c>
       <c r="K44" s="15" t="inlineStr">
         <is>
-          <t>The resolution date must be on or after the onset date and cannot be in the future.</t>
+          <t>The onset date cannot be in the future, and the same event with the same onset date cannot be entered twice for one animal.</t>
         </is>
       </c>
       <c r="N44" s="15" t="inlineStr">
         <is>
-          <t>Enter the date of resolution.</t>
+          <t>Enter the date of onset.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="18">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>is_notifiable</t>
+          <t>date_resolution</t>
         </is>
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>Notifiable Disease</t>
-        </is>
-      </c>
-      <c r="D45" s="15" t="inlineStr">
-        <is>
-          <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
-        </is>
-      </c>
-      <c r="F45" s="15" t="inlineStr">
-        <is>
-          <t>no</t>
+          <t>Date of Resolution</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="G45" s="21" t="inlineStr">
         <is>
-          <t>${event_type} = 'disease'</t>
-        </is>
-      </c>
-      <c r="I45" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
+          <t>${event_type} = 'disease' or ${event_type} = 'injury' or ${event_type} = 'recovery'</t>
+        </is>
+      </c>
+      <c r="J45" s="15" t="inlineStr">
+        <is>
+          <t>(. &gt;= ${date_onset} or ${date_onset} = '') and . &lt;= today()</t>
+        </is>
+      </c>
+      <c r="K45" s="15" t="inlineStr">
+        <is>
+          <t>The resolution date must be on or after the onset date and cannot be in the future.</t>
+        </is>
+      </c>
+      <c r="N45" s="15" t="inlineStr">
+        <is>
+          <t>Enter the date of resolution.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1" s="18">
       <c r="A46" s="15" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>treatment</t>
+          <t>is_notifiable</t>
         </is>
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>Treatment Administered</t>
+          <t>Notifiable Disease</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="G46" s="21" t="inlineStr">
         <is>
-          <t>${event_type} = 'disease' or ${event_type} = 'injury' or ${event_type} = 'treatment'</t>
+          <t>${event_type} = 'disease'</t>
         </is>
       </c>
       <c r="I46" s="15" t="inlineStr">
         <is>
-          <t>multiline</t>
+          <t>minimal</t>
         </is>
       </c>
     </row>
@@ -1865,56 +1855,61 @@
       </c>
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>veterinarian_id</t>
+          <t>treatment</t>
         </is>
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>Veterinarian / Officer</t>
+          <t>Treatment Administered</t>
+        </is>
+      </c>
+      <c r="G47" s="21" t="inlineStr">
+        <is>
+          <t>${event_type} = 'disease' or ${event_type} = 'injury' or ${event_type} = 'treatment'</t>
+        </is>
+      </c>
+      <c r="I47" s="15" t="inlineStr">
+        <is>
+          <t>multiline</t>
         </is>
       </c>
     </row>
     <row r="48" ht="13.5" customHeight="1" s="18">
       <c r="A48" s="15" t="inlineStr">
         <is>
-          <t>select_one location</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>veterinarian_id</t>
         </is>
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="I48" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
+          <t>Veterinarian / Officer</t>
         </is>
       </c>
     </row>
     <row r="49" ht="13.5" customHeight="1" s="18">
       <c r="A49" s="15" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one location</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>location_details</t>
+          <t>location</t>
         </is>
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>Location Details</t>
-        </is>
-      </c>
-      <c r="D49" s="15" t="inlineStr">
-        <is>
-          <t>For example the exact address or the clinic name.</t>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="I49" s="15" t="inlineStr">
+        <is>
+          <t>minimal</t>
         </is>
       </c>
     </row>
@@ -1926,119 +1921,104 @@
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
+          <t>location_details</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>Location Details</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>For example the exact address or the clinic name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="13.5" customFormat="1" customHeight="1" s="19">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
           <t>health_event_notes</t>
         </is>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="D51" s="15" t="inlineStr">
         <is>
           <t>Any additional notes.</t>
         </is>
       </c>
-      <c r="E50" s="15" t="n"/>
-      <c r="F50" s="15" t="n"/>
-      <c r="G50" s="15" t="n"/>
-      <c r="H50" s="15" t="n"/>
-      <c r="I50" s="15" t="inlineStr">
+      <c r="E51" s="15" t="n"/>
+      <c r="F51" s="15" t="n"/>
+      <c r="G51" s="15" t="n"/>
+      <c r="H51" s="15" t="n"/>
+      <c r="I51" s="15" t="inlineStr">
         <is>
           <t>multiline</t>
         </is>
       </c>
-      <c r="J50" s="15" t="n"/>
-      <c r="K50" s="15" t="n"/>
-      <c r="L50" s="15" t="n"/>
-      <c r="M50" s="15" t="n"/>
-    </row>
-    <row r="51" ht="13.5" customFormat="1" customHeight="1" s="19">
-      <c r="A51" s="19" t="inlineStr">
+      <c r="J51" s="15" t="n"/>
+      <c r="K51" s="15" t="n"/>
+      <c r="L51" s="15" t="n"/>
+      <c r="M51" s="15" t="n"/>
+    </row>
+    <row r="52" ht="13.5" customFormat="1" customHeight="1" s="19">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>end_repeat</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="13.5" customFormat="1" customHeight="1" s="19"/>
-    <row r="53" ht="13.5" customHeight="1" s="18">
-      <c r="A53" s="19" t="inlineStr">
+    <row r="53" ht="13.5" customHeight="1" s="18"/>
+    <row r="54" ht="13.5" customFormat="1" customHeight="1" s="15">
+      <c r="A54" s="19" t="inlineStr">
         <is>
           <t>begin_repeat</t>
         </is>
       </c>
-      <c r="B53" s="19" t="inlineStr">
+      <c r="B54" s="19" t="inlineStr">
         <is>
           <t>vaccinations</t>
         </is>
       </c>
-      <c r="C53" s="19" t="inlineStr">
+      <c r="C54" s="19" t="inlineStr">
         <is>
           <t>Vaccinations</t>
         </is>
       </c>
-      <c r="D53" s="19" t="n"/>
-      <c r="E53" s="19" t="n"/>
-      <c r="F53" s="19" t="n"/>
-      <c r="G53" s="19" t="n"/>
-      <c r="H53" s="19" t="n"/>
-      <c r="I53" s="19" t="n"/>
-      <c r="J53" s="19" t="n"/>
-      <c r="K53" s="19" t="n"/>
-      <c r="L53" s="19" t="n"/>
-      <c r="M53" s="19" t="n"/>
-    </row>
-    <row r="54" ht="13.5" customFormat="1" customHeight="1" s="15">
-      <c r="A54" s="15" t="inlineStr">
-        <is>
-          <t>select_one vaccines</t>
-        </is>
-      </c>
-      <c r="B54" s="15" t="inlineStr">
-        <is>
-          <t>vaccine</t>
-        </is>
-      </c>
-      <c r="C54" s="15" t="inlineStr">
-        <is>
-          <t>Vaccine</t>
-        </is>
-      </c>
-      <c r="E54" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I54" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="M54" s="15" t="inlineStr">
-        <is>
-          <t>species = ${species_id}</t>
-        </is>
-      </c>
-      <c r="N54" s="15" t="inlineStr">
-        <is>
-          <t>Select the vaccine.</t>
-        </is>
-      </c>
+      <c r="D54" s="19" t="n"/>
+      <c r="E54" s="19" t="n"/>
+      <c r="F54" s="19" t="n"/>
+      <c r="G54" s="19" t="n"/>
+      <c r="H54" s="19" t="n"/>
+      <c r="I54" s="19" t="n"/>
+      <c r="J54" s="19" t="n"/>
+      <c r="K54" s="19" t="n"/>
+      <c r="L54" s="19" t="n"/>
+      <c r="M54" s="19" t="n"/>
     </row>
     <row r="55" ht="13.5" customHeight="1" s="18">
       <c r="A55" s="15" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one vaccines</t>
         </is>
       </c>
       <c r="B55" s="15" t="inlineStr">
         <is>
-          <t>vaccination_date</t>
+          <t>vaccine</t>
         </is>
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>Vaccination Date</t>
+          <t>Vaccine</t>
         </is>
       </c>
       <c r="E55" s="15" t="inlineStr">
@@ -2046,24 +2026,19 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F55" s="15" t="inlineStr">
-        <is>
-          <t>today()</t>
-        </is>
-      </c>
-      <c r="J55" s="15" t="inlineStr">
-        <is>
-          <t>. &lt;= today()</t>
-        </is>
-      </c>
-      <c r="K55" s="15" t="inlineStr">
-        <is>
-          <t>The vaccination date cannot be in the future, and the same vaccine with the same date cannot be entered twice for one animal.</t>
+      <c r="I55" s="15" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="M55" s="15" t="inlineStr">
+        <is>
+          <t>species = ${species_id}</t>
         </is>
       </c>
       <c r="N55" s="15" t="inlineStr">
         <is>
-          <t>Enter the vaccination date.</t>
+          <t>Select the vaccine.</t>
         </is>
       </c>
     </row>
@@ -2075,39 +2050,64 @@
       </c>
       <c r="B56" s="15" t="inlineStr">
         <is>
-          <t>next_due_date</t>
+          <t>vaccination_date</t>
         </is>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>Next Due Date</t>
+          <t>Vaccination Date</t>
+        </is>
+      </c>
+      <c r="E56" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F56" s="15" t="inlineStr">
+        <is>
+          <t>today()</t>
         </is>
       </c>
       <c r="J56" s="15" t="inlineStr">
         <is>
-          <t>. &gt;= ${vaccination_date} or ${vaccination_date} = ''</t>
+          <t>. &lt;= today()</t>
         </is>
       </c>
       <c r="K56" s="15" t="inlineStr">
         <is>
-          <t>The next due date cannot be before the vaccination date.</t>
+          <t>The vaccination date cannot be in the future, and the same vaccine with the same date cannot be entered twice for one animal.</t>
+        </is>
+      </c>
+      <c r="N56" s="15" t="inlineStr">
+        <is>
+          <t>Enter the vaccination date.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="13.5" customHeight="1" s="18">
       <c r="A57" s="15" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B57" s="15" t="inlineStr">
         <is>
-          <t>batch_number</t>
+          <t>next_due_date</t>
         </is>
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>Batch or Lot Number</t>
+          <t>Next Due Date</t>
+        </is>
+      </c>
+      <c r="J57" s="15" t="inlineStr">
+        <is>
+          <t>. &gt;= ${vaccination_date} or ${vaccination_date} = ''</t>
+        </is>
+      </c>
+      <c r="K57" s="15" t="inlineStr">
+        <is>
+          <t>The next due date cannot be before the vaccination date.</t>
         </is>
       </c>
     </row>
@@ -2119,12 +2119,12 @@
       </c>
       <c r="B58" s="15" t="inlineStr">
         <is>
-          <t>administered_by</t>
+          <t>batch_number</t>
         </is>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Administered By</t>
+          <t>Batch or Lot Number</t>
         </is>
       </c>
     </row>
@@ -2136,124 +2136,99 @@
       </c>
       <c r="B59" s="15" t="inlineStr">
         <is>
+          <t>administered_by</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>Administered By</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="13.5" customFormat="1" customHeight="1" s="19">
+      <c r="A60" s="15" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
           <t>vaccination_notes</t>
         </is>
       </c>
-      <c r="C59" s="15" t="inlineStr">
+      <c r="C60" s="15" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="D59" s="15" t="inlineStr">
+      <c r="D60" s="15" t="inlineStr">
         <is>
           <t>Any notes about this vaccination.</t>
         </is>
       </c>
-      <c r="E59" s="15" t="n"/>
-      <c r="F59" s="15" t="n"/>
-      <c r="G59" s="15" t="n"/>
-      <c r="H59" s="15" t="n"/>
-      <c r="I59" s="15" t="inlineStr">
+      <c r="E60" s="15" t="n"/>
+      <c r="F60" s="15" t="n"/>
+      <c r="G60" s="15" t="n"/>
+      <c r="H60" s="15" t="n"/>
+      <c r="I60" s="15" t="inlineStr">
         <is>
           <t>multiline</t>
         </is>
       </c>
-      <c r="J59" s="15" t="n"/>
-      <c r="K59" s="15" t="n"/>
-      <c r="L59" s="15" t="n"/>
-      <c r="M59" s="15" t="n"/>
-    </row>
-    <row r="60" ht="13.5" customFormat="1" customHeight="1" s="19">
-      <c r="A60" s="19" t="inlineStr">
+      <c r="J60" s="15" t="n"/>
+      <c r="K60" s="15" t="n"/>
+      <c r="L60" s="15" t="n"/>
+      <c r="M60" s="15" t="n"/>
+    </row>
+    <row r="61" ht="13.5" customFormat="1" customHeight="1" s="19">
+      <c r="A61" s="19" t="inlineStr">
         <is>
           <t>end_repeat</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="13.5" customFormat="1" customHeight="1" s="19"/>
-    <row r="62" ht="13.5" customHeight="1" s="18">
-      <c r="A62" s="19" t="inlineStr">
+    <row r="62" ht="13.5" customHeight="1" s="18"/>
+    <row r="63" ht="13.5" customHeight="1" s="18">
+      <c r="A63" s="19" t="inlineStr">
         <is>
           <t>begin_repeat</t>
         </is>
       </c>
-      <c r="B62" s="19" t="inlineStr">
+      <c r="B63" s="19" t="inlineStr">
         <is>
           <t>vital_events</t>
         </is>
       </c>
-      <c r="C62" s="19" t="inlineStr">
+      <c r="C63" s="19" t="inlineStr">
         <is>
           <t>Vital Events</t>
         </is>
       </c>
-      <c r="D62" s="19" t="n"/>
-      <c r="E62" s="19" t="n"/>
-      <c r="F62" s="19" t="n"/>
-      <c r="G62" s="19" t="n"/>
-      <c r="H62" s="19" t="n"/>
-      <c r="I62" s="19" t="n"/>
-      <c r="J62" s="19" t="n"/>
-      <c r="K62" s="19" t="n"/>
-      <c r="L62" s="19" t="n"/>
-      <c r="M62" s="19" t="n"/>
-    </row>
-    <row r="63" ht="13.5" customHeight="1" s="18">
-      <c r="A63" s="15" t="inlineStr">
-        <is>
-          <t>select_one vital_event_type</t>
-        </is>
-      </c>
-      <c r="B63" s="15" t="inlineStr">
-        <is>
-          <t>vital_event_type</t>
-        </is>
-      </c>
-      <c r="C63" s="15" t="inlineStr">
-        <is>
-          <t>Event Type</t>
-        </is>
-      </c>
-      <c r="E63" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I63" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="J63" s="15" t="inlineStr">
-        <is>
-          <t>not(. = 'mortality') or count(../../vital_events[vital_event_type = 'mortality']) = 1</t>
-        </is>
-      </c>
-      <c r="K63" s="15" t="inlineStr">
-        <is>
-          <t>Only one death (mortality) event can be recorded for each animal.</t>
-        </is>
-      </c>
-      <c r="N63" s="15" t="inlineStr">
-        <is>
-          <t>Select the event type.</t>
-        </is>
-      </c>
+      <c r="D63" s="19" t="n"/>
+      <c r="E63" s="19" t="n"/>
+      <c r="F63" s="19" t="n"/>
+      <c r="G63" s="19" t="n"/>
+      <c r="H63" s="19" t="n"/>
+      <c r="I63" s="19" t="n"/>
+      <c r="J63" s="19" t="n"/>
+      <c r="K63" s="19" t="n"/>
+      <c r="L63" s="19" t="n"/>
+      <c r="M63" s="19" t="n"/>
     </row>
     <row r="64" ht="13.5" customHeight="1" s="18">
       <c r="A64" s="15" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one vital_event_type</t>
         </is>
       </c>
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>vital_event_type</t>
         </is>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>Event Date</t>
+          <t>Event Type</t>
         </is>
       </c>
       <c r="E64" s="15" t="inlineStr">
@@ -2261,63 +2236,88 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F64" s="15" t="inlineStr">
-        <is>
-          <t>today()</t>
+      <c r="I64" s="15" t="inlineStr">
+        <is>
+          <t>minimal</t>
         </is>
       </c>
       <c r="J64" s="15" t="inlineStr">
         <is>
-          <t>. &lt;= today()</t>
+          <t>not(. = 'mortality') or count(../../vital_events[vital_event_type = 'mortality']) = 1</t>
         </is>
       </c>
       <c r="K64" s="15" t="inlineStr">
         <is>
-          <t>The event date cannot be in the future.</t>
+          <t>Only one death (mortality) event can be recorded for each animal.</t>
         </is>
       </c>
       <c r="N64" s="15" t="inlineStr">
         <is>
-          <t>Enter the event date.</t>
+          <t>Select the event type.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="13.5" customHeight="1" s="18">
       <c r="A65" s="15" t="inlineStr">
         <is>
-          <t>select_one location</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B65" s="15" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="I65" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
+          <t>Event Date</t>
+        </is>
+      </c>
+      <c r="E65" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F65" s="15" t="inlineStr">
+        <is>
+          <t>today()</t>
+        </is>
+      </c>
+      <c r="J65" s="15" t="inlineStr">
+        <is>
+          <t>. &lt;= today()</t>
+        </is>
+      </c>
+      <c r="K65" s="15" t="inlineStr">
+        <is>
+          <t>The event date cannot be in the future.</t>
+        </is>
+      </c>
+      <c r="N65" s="15" t="inlineStr">
+        <is>
+          <t>Enter the event date.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="13.5" customHeight="1" s="18">
       <c r="A66" s="15" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one location</t>
         </is>
       </c>
       <c r="B66" s="15" t="inlineStr">
         <is>
-          <t>location_details</t>
+          <t>location</t>
         </is>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>Location Details</t>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="I66" s="15" t="inlineStr">
+        <is>
+          <t>minimal</t>
         </is>
       </c>
     </row>
@@ -2329,17 +2329,12 @@
       </c>
       <c r="B67" s="15" t="inlineStr">
         <is>
-          <t>reporting_officer_id</t>
+          <t>location_details</t>
         </is>
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>Reporting Officer</t>
-        </is>
-      </c>
-      <c r="F67" s="15" t="inlineStr">
-        <is>
-          <t>Administrator</t>
+          <t>Location Details</t>
         </is>
       </c>
     </row>
@@ -2351,224 +2346,219 @@
       </c>
       <c r="B68" s="15" t="inlineStr">
         <is>
+          <t>reporting_officer_id</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>Reporting Officer</t>
+        </is>
+      </c>
+      <c r="F68" s="15" t="inlineStr">
+        <is>
+          <t>Administrator</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="13.5" customFormat="1" customHeight="1" s="19">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
           <t>vital_event_details</t>
         </is>
       </c>
-      <c r="C68" s="15" t="inlineStr">
+      <c r="C69" s="15" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="I68" s="15" t="inlineStr">
+      <c r="I69" s="15" t="inlineStr">
         <is>
           <t>multiline</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="13.5" customFormat="1" customHeight="1" s="19">
-      <c r="A69" s="15" t="n"/>
-      <c r="B69" s="15" t="n"/>
-      <c r="C69" s="15" t="n"/>
-      <c r="D69" s="15" t="n"/>
-      <c r="E69" s="15" t="n"/>
-      <c r="F69" s="15" t="n"/>
-      <c r="G69" s="15" t="n"/>
-      <c r="H69" s="15" t="n"/>
-      <c r="I69" s="15" t="n"/>
-      <c r="J69" s="15" t="n"/>
-      <c r="K69" s="15" t="n"/>
-      <c r="L69" s="15" t="n"/>
-      <c r="M69" s="15" t="n"/>
-    </row>
     <row r="70" ht="15" customHeight="1" s="18">
-      <c r="A70" s="19" t="inlineStr">
+      <c r="A70" s="15" t="n"/>
+      <c r="B70" s="15" t="n"/>
+      <c r="C70" s="15" t="n"/>
+      <c r="D70" s="15" t="n"/>
+      <c r="E70" s="15" t="n"/>
+      <c r="F70" s="15" t="n"/>
+      <c r="G70" s="15" t="n"/>
+      <c r="H70" s="15" t="n"/>
+      <c r="I70" s="15" t="n"/>
+      <c r="J70" s="15" t="n"/>
+      <c r="K70" s="15" t="n"/>
+      <c r="L70" s="15" t="n"/>
+      <c r="M70" s="15" t="n"/>
+    </row>
+    <row r="71" ht="13.5" customHeight="1" s="18">
+      <c r="A71" s="19" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B70" s="19" t="inlineStr">
+      <c r="B71" s="19" t="inlineStr">
         <is>
           <t>birth_details</t>
         </is>
       </c>
-      <c r="C70" s="19" t="inlineStr">
+      <c r="C71" s="19" t="inlineStr">
         <is>
           <t>Birth Details</t>
         </is>
       </c>
-      <c r="D70" s="19" t="n"/>
-      <c r="E70" s="19" t="n"/>
-      <c r="F70" s="19" t="n"/>
-      <c r="G70" s="21" t="inlineStr">
+      <c r="D71" s="19" t="n"/>
+      <c r="E71" s="19" t="n"/>
+      <c r="F71" s="19" t="n"/>
+      <c r="G71" s="21" t="inlineStr">
         <is>
           <t>${vital_event_type} = 'birth'</t>
         </is>
       </c>
-      <c r="H70" s="19" t="n"/>
-      <c r="I70" s="19" t="n"/>
-      <c r="J70" s="19" t="n"/>
-      <c r="K70" s="19" t="n"/>
-      <c r="L70" s="19" t="n"/>
-      <c r="M70" s="19" t="n"/>
-    </row>
-    <row r="71" ht="13.5" customHeight="1" s="18">
-      <c r="A71" s="15" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="B71" s="15" t="inlineStr">
-        <is>
-          <t>offspring_count</t>
-        </is>
-      </c>
-      <c r="C71" s="15" t="inlineStr">
-        <is>
-          <t>Number of Offspring</t>
-        </is>
-      </c>
-      <c r="E71" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J71" s="15" t="inlineStr">
-        <is>
-          <t>. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="K71" s="15" t="inlineStr">
-        <is>
-          <t>Enter 0 or more offspring.</t>
-        </is>
-      </c>
-      <c r="N71" s="15" t="inlineStr">
-        <is>
-          <t>Enter the number of offspring.</t>
-        </is>
-      </c>
+      <c r="H71" s="19" t="n"/>
+      <c r="I71" s="19" t="n"/>
+      <c r="J71" s="19" t="n"/>
+      <c r="K71" s="19" t="n"/>
+      <c r="L71" s="19" t="n"/>
+      <c r="M71" s="19" t="n"/>
     </row>
     <row r="72" ht="13.5" customHeight="1" s="18">
       <c r="A72" s="15" t="inlineStr">
         <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>offspring_count</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="inlineStr">
+        <is>
+          <t>Number of Offspring</t>
+        </is>
+      </c>
+      <c r="E72" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J72" s="15" t="inlineStr">
+        <is>
+          <t>. &gt;= 0</t>
+        </is>
+      </c>
+      <c r="K72" s="15" t="inlineStr">
+        <is>
+          <t>Enter 0 or more offspring.</t>
+        </is>
+      </c>
+      <c r="N72" s="15" t="inlineStr">
+        <is>
+          <t>Enter the number of offspring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="13.5" customFormat="1" customHeight="1" s="19">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
           <t>select_one gender_offspring</t>
         </is>
       </c>
-      <c r="B72" s="15" t="inlineStr">
+      <c r="B73" s="15" t="inlineStr">
         <is>
           <t>sex_of_offspring</t>
         </is>
       </c>
-      <c r="C72" s="15" t="inlineStr">
+      <c r="C73" s="15" t="inlineStr">
         <is>
           <t>Sex of Offspring</t>
         </is>
       </c>
-      <c r="E72" s="15" t="inlineStr">
+      <c r="E73" s="15" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="N72" s="15" t="inlineStr">
+      <c r="N73" s="15" t="inlineStr">
         <is>
           <t>Select the sex of offspring.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="13.5" customFormat="1" customHeight="1" s="19">
-      <c r="A73" s="19" t="inlineStr">
-        <is>
-          <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customFormat="1" customHeight="1" s="15">
       <c r="A74" s="19" t="inlineStr">
         <is>
+          <t>end_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="13.5" customFormat="1" customHeight="1" s="15">
+      <c r="A75" s="19" t="inlineStr">
+        <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B74" s="19" t="inlineStr">
+      <c r="B75" s="19" t="inlineStr">
         <is>
           <t>disease_details</t>
         </is>
       </c>
-      <c r="C74" s="19" t="inlineStr">
+      <c r="C75" s="19" t="inlineStr">
         <is>
           <t>Disease Details</t>
         </is>
       </c>
-      <c r="D74" s="19" t="n"/>
-      <c r="E74" s="19" t="n"/>
-      <c r="F74" s="19" t="n"/>
-      <c r="G74" s="21" t="inlineStr">
+      <c r="D75" s="19" t="n"/>
+      <c r="E75" s="19" t="n"/>
+      <c r="F75" s="19" t="n"/>
+      <c r="G75" s="21" t="inlineStr">
         <is>
           <t>${vital_event_type} = 'disease'</t>
         </is>
       </c>
-      <c r="H74" s="19" t="n"/>
-      <c r="I74" s="19" t="n"/>
-      <c r="J74" s="19" t="n"/>
-      <c r="K74" s="19" t="n"/>
-      <c r="L74" s="19" t="n"/>
-      <c r="M74" s="19" t="n"/>
-    </row>
-    <row r="75" ht="13.5" customFormat="1" customHeight="1" s="15">
-      <c r="A75" s="15" t="inlineStr">
-        <is>
-          <t>select_one disease</t>
-        </is>
-      </c>
-      <c r="B75" s="15" t="inlineStr">
-        <is>
-          <t>disease_type</t>
-        </is>
-      </c>
-      <c r="C75" s="15" t="inlineStr">
-        <is>
-          <t>Disease / Diagnosis</t>
-        </is>
-      </c>
-      <c r="E75" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I75" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="N75" s="15" t="inlineStr">
-        <is>
-          <t>Select the disease / diagnosis.</t>
-        </is>
-      </c>
+      <c r="H75" s="19" t="n"/>
+      <c r="I75" s="19" t="n"/>
+      <c r="J75" s="19" t="n"/>
+      <c r="K75" s="19" t="n"/>
+      <c r="L75" s="19" t="n"/>
+      <c r="M75" s="19" t="n"/>
     </row>
     <row r="76" ht="13.5" customFormat="1" customHeight="1" s="15">
       <c r="A76" s="15" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one disease</t>
         </is>
       </c>
       <c r="B76" s="15" t="inlineStr">
         <is>
-          <t>vital_date_onset</t>
+          <t>disease_type</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>Date of Onset</t>
-        </is>
-      </c>
-      <c r="J76" s="15" t="inlineStr">
-        <is>
-          <t>. &lt;= today()</t>
-        </is>
-      </c>
-      <c r="K76" s="15" t="inlineStr">
-        <is>
-          <t>The onset date cannot be in the future, and the same disease with the same onset date cannot be entered twice for one animal.</t>
+          <t>Disease / Diagnosis</t>
+        </is>
+      </c>
+      <c r="E76" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I76" s="15" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="N76" s="15" t="inlineStr">
+        <is>
+          <t>Select the disease / diagnosis.</t>
         </is>
       </c>
     </row>
@@ -2580,61 +2570,71 @@
       </c>
       <c r="B77" s="15" t="inlineStr">
         <is>
-          <t>vital_date_resolution</t>
+          <t>vital_date_onset</t>
         </is>
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>Date of Resolution</t>
+          <t>Date of Onset</t>
         </is>
       </c>
       <c r="J77" s="15" t="inlineStr">
         <is>
-          <t>(. &gt;= ${vital_date_onset} or ${vital_date_onset} = '') and . &lt;= today()</t>
+          <t>. &lt;= today()</t>
         </is>
       </c>
       <c r="K77" s="15" t="inlineStr">
         <is>
-          <t>The resolution date must be on or after the onset date and cannot be in the future.</t>
+          <t>The onset date cannot be in the future, and the same disease with the same onset date cannot be entered twice for one animal.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="13.5" customFormat="1" customHeight="1" s="15">
       <c r="A78" s="15" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B78" s="15" t="inlineStr">
         <is>
-          <t>vital_is_notifiable</t>
+          <t>vital_date_resolution</t>
         </is>
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>Notifiable Disease</t>
-        </is>
-      </c>
-      <c r="D78" s="15" t="inlineStr">
-        <is>
-          <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
+          <t>Date of Resolution</t>
+        </is>
+      </c>
+      <c r="J78" s="15" t="inlineStr">
+        <is>
+          <t>(. &gt;= ${vital_date_onset} or ${vital_date_onset} = '') and . &lt;= today()</t>
+        </is>
+      </c>
+      <c r="K78" s="15" t="inlineStr">
+        <is>
+          <t>The resolution date must be on or after the onset date and cannot be in the future.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="13.5" customFormat="1" customHeight="1" s="15">
       <c r="A79" s="15" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B79" s="15" t="inlineStr">
         <is>
-          <t>treatment</t>
+          <t>vital_is_notifiable</t>
         </is>
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>Treatment Administered</t>
+          <t>Notifiable Disease</t>
+        </is>
+      </c>
+      <c r="D79" s="15" t="inlineStr">
+        <is>
+          <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
         </is>
       </c>
     </row>
@@ -2646,190 +2646,165 @@
       </c>
       <c r="B80" s="15" t="inlineStr">
         <is>
-          <t>veterinarian_id</t>
+          <t>treatment</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>Attending Veterinarian</t>
+          <t>Treatment Administered</t>
         </is>
       </c>
     </row>
     <row r="81" ht="13.5" customFormat="1" customHeight="1" s="19">
       <c r="A81" s="15" t="inlineStr">
         <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="inlineStr">
+        <is>
+          <t>veterinarian_id</t>
+        </is>
+      </c>
+      <c r="C81" s="15" t="inlineStr">
+        <is>
+          <t>Attending Veterinarian</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="13.5" customHeight="1" s="18">
+      <c r="A82" s="15" t="inlineStr">
+        <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B81" s="15" t="inlineStr">
+      <c r="B82" s="15" t="inlineStr">
         <is>
           <t>is_notifiable</t>
         </is>
       </c>
-      <c r="C81" s="15" t="inlineStr">
+      <c r="C82" s="15" t="inlineStr">
         <is>
           <t>Notifiable Disease</t>
         </is>
       </c>
-      <c r="D81" s="15" t="inlineStr">
+      <c r="D82" s="15" t="inlineStr">
         <is>
           <t>Choose Yes if this disease must be reported to the veterinary authorities.</t>
         </is>
       </c>
-      <c r="E81" s="15" t="n"/>
-      <c r="F81" s="15" t="n"/>
-      <c r="G81" s="15" t="n"/>
-      <c r="H81" s="15" t="n"/>
-      <c r="I81" s="15" t="n"/>
-      <c r="J81" s="15" t="n"/>
-      <c r="K81" s="15" t="n"/>
-      <c r="L81" s="15" t="n"/>
-      <c r="M81" s="15" t="n"/>
-    </row>
-    <row r="82" ht="13.5" customHeight="1" s="18">
-      <c r="A82" s="19" t="inlineStr">
+      <c r="E82" s="15" t="n"/>
+      <c r="F82" s="15" t="n"/>
+      <c r="G82" s="15" t="n"/>
+      <c r="H82" s="15" t="n"/>
+      <c r="I82" s="15" t="n"/>
+      <c r="J82" s="15" t="n"/>
+      <c r="K82" s="15" t="n"/>
+      <c r="L82" s="15" t="n"/>
+      <c r="M82" s="15" t="n"/>
+    </row>
+    <row r="83" ht="15" customFormat="1" customHeight="1" s="19">
+      <c r="A83" s="19" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
       </c>
-      <c r="B82" s="19" t="n"/>
-      <c r="C82" s="19" t="n"/>
-      <c r="D82" s="19" t="n"/>
-      <c r="E82" s="19" t="n"/>
-      <c r="F82" s="19" t="n"/>
-      <c r="G82" s="19" t="n"/>
-      <c r="H82" s="19" t="n"/>
-      <c r="I82" s="19" t="n"/>
-      <c r="J82" s="19" t="n"/>
-      <c r="K82" s="19" t="n"/>
-      <c r="L82" s="19" t="n"/>
-      <c r="M82" s="19" t="n"/>
-    </row>
-    <row r="83" ht="15" customFormat="1" customHeight="1" s="19">
-      <c r="A83" s="15" t="inlineStr">
+      <c r="B83" s="19" t="n"/>
+      <c r="C83" s="19" t="n"/>
+      <c r="D83" s="19" t="n"/>
+      <c r="E83" s="19" t="n"/>
+      <c r="F83" s="19" t="n"/>
+      <c r="G83" s="19" t="n"/>
+      <c r="H83" s="19" t="n"/>
+      <c r="I83" s="19" t="n"/>
+      <c r="J83" s="19" t="n"/>
+      <c r="K83" s="19" t="n"/>
+      <c r="L83" s="19" t="n"/>
+      <c r="M83" s="19" t="n"/>
+    </row>
+    <row r="84" ht="13.5" customFormat="1" customHeight="1" s="19">
+      <c r="A84" s="15" t="inlineStr">
         <is>
           <t>select_one cause_of_event</t>
         </is>
       </c>
-      <c r="B83" s="15" t="inlineStr">
+      <c r="B84" s="15" t="inlineStr">
         <is>
           <t>cause</t>
         </is>
       </c>
-      <c r="C83" s="15" t="inlineStr">
+      <c r="C84" s="15" t="inlineStr">
         <is>
           <t>Cause</t>
         </is>
       </c>
-      <c r="D83" s="15" t="n"/>
-      <c r="E83" s="15" t="n"/>
-      <c r="F83" s="15" t="n"/>
-      <c r="G83" s="21" t="inlineStr">
+      <c r="D84" s="15" t="n"/>
+      <c r="E84" s="15" t="n"/>
+      <c r="F84" s="15" t="n"/>
+      <c r="G84" s="21" t="inlineStr">
         <is>
           <t>${vital_event_type} = 'mortality'</t>
         </is>
       </c>
-      <c r="H83" s="15" t="n"/>
-      <c r="I83" s="15" t="inlineStr">
+      <c r="H84" s="15" t="n"/>
+      <c r="I84" s="15" t="inlineStr">
         <is>
           <t>minimal</t>
         </is>
       </c>
-      <c r="J83" s="15" t="n"/>
-      <c r="K83" s="15" t="n"/>
-      <c r="L83" s="15" t="n"/>
-      <c r="M83" s="15" t="n"/>
-    </row>
-    <row r="84" ht="13.5" customFormat="1" customHeight="1" s="19">
-      <c r="A84" s="19" t="inlineStr">
+      <c r="J84" s="15" t="n"/>
+      <c r="K84" s="15" t="n"/>
+      <c r="L84" s="15" t="n"/>
+      <c r="M84" s="15" t="n"/>
+    </row>
+    <row r="85" ht="13.5" customFormat="1" customHeight="1" s="19">
+      <c r="A85" s="19" t="inlineStr">
         <is>
           <t>end_repeat</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="13.5" customFormat="1" customHeight="1" s="19"/>
-    <row r="86" ht="13.5" customHeight="1" s="18">
-      <c r="A86" s="19" t="inlineStr">
+    <row r="86" ht="13.5" customHeight="1" s="18"/>
+    <row r="87" ht="13.5" customHeight="1" s="18">
+      <c r="A87" s="19" t="inlineStr">
         <is>
           <t>begin_repeat</t>
         </is>
       </c>
-      <c r="B86" s="19" t="inlineStr">
+      <c r="B87" s="19" t="inlineStr">
         <is>
           <t>breeding_events</t>
         </is>
       </c>
-      <c r="C86" s="19" t="inlineStr">
+      <c r="C87" s="19" t="inlineStr">
         <is>
           <t>Breeding Events</t>
         </is>
       </c>
-      <c r="D86" s="19" t="n"/>
-      <c r="E86" s="19" t="n"/>
-      <c r="F86" s="19" t="n"/>
-      <c r="H86" s="19" t="n"/>
-      <c r="I86" s="19" t="n"/>
-      <c r="J86" s="19" t="n"/>
-      <c r="K86" s="19" t="n"/>
-      <c r="L86" s="19" t="n"/>
-      <c r="M86" s="19" t="n"/>
-    </row>
-    <row r="87" ht="13.5" customHeight="1" s="18">
-      <c r="A87" s="15" t="inlineStr">
-        <is>
-          <t>select_one breeding_event_type</t>
-        </is>
-      </c>
-      <c r="B87" s="15" t="inlineStr">
-        <is>
-          <t>breeding_event_type</t>
-        </is>
-      </c>
-      <c r="C87" s="15" t="inlineStr">
-        <is>
-          <t>Breeding Type</t>
-        </is>
-      </c>
-      <c r="E87" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I87" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="J87" s="15" t="inlineStr">
-        <is>
-          <t>../../gender = 'female'</t>
-        </is>
-      </c>
-      <c r="K87" s="15" t="inlineStr">
-        <is>
-          <t>Only female animals can have breeding events. Check the sex recorded for this animal.</t>
-        </is>
-      </c>
-      <c r="N87" s="15" t="inlineStr">
-        <is>
-          <t>Select the breeding type.</t>
-        </is>
-      </c>
+      <c r="D87" s="19" t="n"/>
+      <c r="E87" s="19" t="n"/>
+      <c r="F87" s="19" t="n"/>
+      <c r="H87" s="19" t="n"/>
+      <c r="I87" s="19" t="n"/>
+      <c r="J87" s="19" t="n"/>
+      <c r="K87" s="19" t="n"/>
+      <c r="L87" s="19" t="n"/>
+      <c r="M87" s="19" t="n"/>
     </row>
     <row r="88" ht="13.5" customHeight="1" s="18">
       <c r="A88" s="15" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one breeding_event_type</t>
         </is>
       </c>
       <c r="B88" s="15" t="inlineStr">
         <is>
-          <t>breeding_date</t>
+          <t>breeding_event_type</t>
         </is>
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Breeding Date</t>
+          <t>Breeding Type</t>
         </is>
       </c>
       <c r="E88" s="15" t="inlineStr">
@@ -2837,63 +2812,88 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F88" s="15" t="inlineStr">
-        <is>
-          <t>today()</t>
+      <c r="I88" s="15" t="inlineStr">
+        <is>
+          <t>minimal</t>
         </is>
       </c>
       <c r="J88" s="15" t="inlineStr">
         <is>
-          <t>. &lt;= today()</t>
+          <t>../../gender = 'female'</t>
         </is>
       </c>
       <c r="K88" s="15" t="inlineStr">
         <is>
-          <t>The breeding date cannot be in the future, and the same breeding event with the same date cannot be entered twice for one animal.</t>
+          <t>Only female animals can have breeding events. Check the sex recorded for this animal.</t>
         </is>
       </c>
       <c r="N88" s="15" t="inlineStr">
         <is>
-          <t>Enter the breeding date.</t>
+          <t>Select the breeding type.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="13.5" customHeight="1" s="18">
       <c r="A89" s="15" t="inlineStr">
         <is>
-          <t>select_one location</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B89" s="15" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>breeding_date</t>
         </is>
       </c>
       <c r="C89" s="15" t="inlineStr">
         <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="I89" s="15" t="inlineStr">
-        <is>
-          <t>minimal</t>
+          <t>Breeding Date</t>
+        </is>
+      </c>
+      <c r="E89" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F89" s="15" t="inlineStr">
+        <is>
+          <t>today()</t>
+        </is>
+      </c>
+      <c r="J89" s="15" t="inlineStr">
+        <is>
+          <t>. &lt;= today()</t>
+        </is>
+      </c>
+      <c r="K89" s="15" t="inlineStr">
+        <is>
+          <t>The breeding date cannot be in the future, and the same breeding event with the same date cannot be entered twice for one animal.</t>
+        </is>
+      </c>
+      <c r="N89" s="15" t="inlineStr">
+        <is>
+          <t>Enter the breeding date.</t>
         </is>
       </c>
     </row>
     <row r="90" ht="13.5" customHeight="1" s="18">
       <c r="A90" s="15" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one location</t>
         </is>
       </c>
       <c r="B90" s="15" t="inlineStr">
         <is>
-          <t>location_details</t>
+          <t>location</t>
         </is>
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>Location Details</t>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="I90" s="15" t="inlineStr">
+        <is>
+          <t>minimal</t>
         </is>
       </c>
     </row>
@@ -2905,29 +2905,29 @@
       </c>
       <c r="B91" s="15" t="inlineStr">
         <is>
-          <t>sire_or_semen_id</t>
+          <t>location_details</t>
         </is>
       </c>
       <c r="C91" s="15" t="inlineStr">
         <is>
-          <t>Sire / Semen Source</t>
+          <t>Location Details</t>
         </is>
       </c>
     </row>
     <row r="92" ht="72.75" customHeight="1" s="18">
       <c r="A92" s="15" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B92" s="15" t="inlineStr">
         <is>
-          <t>gestation_days</t>
-        </is>
-      </c>
-      <c r="H92" s="21" t="inlineStr">
-        <is>
-          <t>if(${species_id} = 'cattle', 283, if(${species_id} = 'goat', 150, if(${species_id} = 'sheep', 150, if(${species_id} = 'camel', 390, if(selected(${species_id}, 'horse') or selected(${species_id}, 'donkey') or selected(${species_id}, 'mule'), 340, if(${species_id} = 'poultry', 21, 280))))))</t>
+          <t>sire_or_semen_id</t>
+        </is>
+      </c>
+      <c r="C92" s="15" t="inlineStr">
+        <is>
+          <t>Sire / Semen Source</t>
         </is>
       </c>
     </row>
@@ -2939,202 +2939,192 @@
       </c>
       <c r="B93" s="15" t="inlineStr">
         <is>
-          <t>expected_calving_date_calc</t>
+          <t>gestation_days</t>
         </is>
       </c>
       <c r="H93" s="21" t="inlineStr">
         <is>
-          <t>${breeding_date} + ${gestation_days}</t>
+          <t>if(${species_id} = 'cattle', 283, if(${species_id} = 'goat', 150, if(${species_id} = 'sheep', 150, if(${species_id} = 'camel', 390, if(selected(${species_id}, 'horse') or selected(${species_id}, 'donkey') or selected(${species_id}, 'mule'), 340, if(${species_id} = 'poultry', 21, 280))))))</t>
         </is>
       </c>
     </row>
     <row r="94" ht="13.5" customHeight="1" s="18">
       <c r="A94" s="15" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B94" s="15" t="inlineStr">
         <is>
-          <t>expected_calving_date</t>
-        </is>
-      </c>
-      <c r="C94" s="15" t="inlineStr">
-        <is>
-          <t>Expected Calving Date</t>
-        </is>
-      </c>
-      <c r="J94" s="15" t="inlineStr">
-        <is>
-          <t>. &gt;= ${breeding_date}</t>
-        </is>
-      </c>
-      <c r="K94" s="15" t="inlineStr">
-        <is>
-          <t>The expected calving date cannot be before the breeding date.</t>
+          <t>expected_calving_date_calc</t>
+        </is>
+      </c>
+      <c r="H94" s="21" t="inlineStr">
+        <is>
+          <t>${breeding_date} + ${gestation_days}</t>
         </is>
       </c>
     </row>
     <row r="95" ht="13.5" customHeight="1" s="18">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t>select_one pregnancy</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B95" s="15" t="inlineStr">
         <is>
-          <t>pregnancy_confirmed</t>
+          <t>expected_calving_date</t>
         </is>
       </c>
       <c r="C95" s="15" t="inlineStr">
         <is>
-          <t>Pregnancy Confirmed</t>
+          <t>Expected Calving Date</t>
+        </is>
+      </c>
+      <c r="J95" s="15" t="inlineStr">
+        <is>
+          <t>. &gt;= ${breeding_date}</t>
+        </is>
+      </c>
+      <c r="K95" s="15" t="inlineStr">
+        <is>
+          <t>The expected calving date cannot be before the breeding date.</t>
         </is>
       </c>
     </row>
     <row r="96" ht="13.5" customHeight="1" s="18">
       <c r="A96" s="15" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one pregnancy</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
         <is>
-          <t>pregnancy_confirmation_date</t>
+          <t>pregnancy_confirmed</t>
         </is>
       </c>
       <c r="C96" s="15" t="inlineStr">
         <is>
-          <t>Pregnancy Confirmation Date</t>
-        </is>
-      </c>
-      <c r="G96" s="15" t="inlineStr">
-        <is>
-          <t>${pregnancy_confirmed} = 'yes'</t>
-        </is>
-      </c>
-      <c r="J96" s="15" t="inlineStr">
-        <is>
-          <t>. &lt;= today()</t>
-        </is>
-      </c>
-      <c r="K96" s="15" t="inlineStr">
-        <is>
-          <t>The pregnancy confirmation date cannot be in the future.</t>
+          <t>Pregnancy Confirmed</t>
         </is>
       </c>
     </row>
     <row r="97" ht="13.5" customHeight="1" s="18">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>select_one outcome</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B97" s="15" t="inlineStr">
         <is>
-          <t>outcome</t>
+          <t>pregnancy_confirmation_date</t>
         </is>
       </c>
       <c r="C97" s="15" t="inlineStr">
         <is>
-          <t>Outcome</t>
+          <t>Pregnancy Confirmation Date</t>
         </is>
       </c>
       <c r="G97" s="15" t="inlineStr">
         <is>
-          <t>${expected_calving_date} != ''</t>
-        </is>
-      </c>
-      <c r="H97" s="21" t="n"/>
+          <t>${pregnancy_confirmed} = 'yes'</t>
+        </is>
+      </c>
+      <c r="J97" s="15" t="inlineStr">
+        <is>
+          <t>. &lt;= today()</t>
+        </is>
+      </c>
+      <c r="K97" s="15" t="inlineStr">
+        <is>
+          <t>The pregnancy confirmation date cannot be in the future.</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="13.5" customFormat="1" customHeight="1" s="19">
       <c r="A98" s="15" t="inlineStr">
         <is>
+          <t>select_one outcome</t>
+        </is>
+      </c>
+      <c r="B98" s="15" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="C98" s="15" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="G98" s="15" t="inlineStr">
+        <is>
+          <t>${expected_calving_date} != ''</t>
+        </is>
+      </c>
+      <c r="H98" s="21" t="n"/>
+    </row>
+    <row r="99" ht="13.5" customHeight="1" s="18">
+      <c r="A99" s="15" t="inlineStr">
+        <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B98" s="15" t="inlineStr">
+      <c r="B99" s="15" t="inlineStr">
         <is>
           <t>breeding_notes</t>
         </is>
       </c>
-      <c r="C98" s="15" t="inlineStr">
+      <c r="C99" s="15" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="D98" s="15" t="n"/>
-      <c r="E98" s="15" t="n"/>
-      <c r="F98" s="15" t="n"/>
-      <c r="G98" s="15" t="n"/>
-      <c r="H98" s="15" t="n"/>
-      <c r="I98" s="15" t="inlineStr">
+      <c r="D99" s="15" t="n"/>
+      <c r="E99" s="15" t="n"/>
+      <c r="F99" s="15" t="n"/>
+      <c r="G99" s="15" t="n"/>
+      <c r="H99" s="15" t="n"/>
+      <c r="I99" s="15" t="inlineStr">
         <is>
           <t>multiline</t>
         </is>
       </c>
-      <c r="J98" s="15" t="n"/>
-      <c r="K98" s="15" t="n"/>
-      <c r="L98" s="15" t="n"/>
-      <c r="M98" s="15" t="n"/>
-    </row>
-    <row r="99" ht="13.5" customHeight="1" s="18">
-      <c r="A99" s="19" t="inlineStr">
+      <c r="J99" s="15" t="n"/>
+      <c r="K99" s="15" t="n"/>
+      <c r="L99" s="15" t="n"/>
+      <c r="M99" s="15" t="n"/>
+    </row>
+    <row r="100" ht="13.5" customHeight="1" s="18">
+      <c r="A100" s="19" t="inlineStr">
         <is>
           <t>begin_group</t>
         </is>
       </c>
-      <c r="B99" s="19" t="inlineStr">
+      <c r="B100" s="19" t="inlineStr">
         <is>
           <t>artificial_insemination_tab</t>
         </is>
       </c>
-      <c r="C99" s="19" t="inlineStr">
+      <c r="C100" s="19" t="inlineStr">
         <is>
           <t>Artificial Insemination Details</t>
         </is>
       </c>
-      <c r="D99" s="19" t="n"/>
-      <c r="E99" s="19" t="n"/>
-      <c r="F99" s="19" t="n"/>
-      <c r="G99" s="15" t="inlineStr">
+      <c r="D100" s="19" t="n"/>
+      <c r="E100" s="19" t="n"/>
+      <c r="F100" s="19" t="n"/>
+      <c r="G100" s="15" t="inlineStr">
         <is>
           <t>${breeding_event_type} = 'artificial_insemination'</t>
         </is>
       </c>
-      <c r="H99" s="19" t="n"/>
-      <c r="I99" s="19" t="n"/>
-      <c r="J99" s="19" t="n"/>
-      <c r="K99" s="19" t="n"/>
-      <c r="L99" s="19" t="n"/>
-      <c r="M99" s="19" t="n"/>
-    </row>
-    <row r="100" ht="13.5" customHeight="1" s="18">
-      <c r="A100" s="15" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B100" s="15" t="inlineStr">
-        <is>
-          <t>ai_technician_id</t>
-        </is>
-      </c>
-      <c r="C100" s="15" t="inlineStr">
-        <is>
-          <t>Artificial Insemination Technician</t>
-        </is>
-      </c>
-      <c r="E100" s="15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="N100" s="15" t="inlineStr">
-        <is>
-          <t>Enter the name or ID of the artificial insemination technician.</t>
-        </is>
-      </c>
+      <c r="H100" s="19" t="n"/>
+      <c r="I100" s="19" t="n"/>
+      <c r="J100" s="19" t="n"/>
+      <c r="K100" s="19" t="n"/>
+      <c r="L100" s="19" t="n"/>
+      <c r="M100" s="19" t="n"/>
     </row>
     <row r="101" ht="13.5" customHeight="1" s="18">
       <c r="A101" s="15" t="inlineStr">
@@ -3144,12 +3134,22 @@
       </c>
       <c r="B101" s="15" t="inlineStr">
         <is>
-          <t>ai_technique</t>
+          <t>ai_technician_id</t>
         </is>
       </c>
       <c r="C101" s="15" t="inlineStr">
         <is>
-          <t>Technique Used</t>
+          <t>Artificial Insemination Technician</t>
+        </is>
+      </c>
+      <c r="E101" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N101" s="15" t="inlineStr">
+        <is>
+          <t>Enter the name or ID of the artificial insemination technician.</t>
         </is>
       </c>
     </row>
@@ -3161,60 +3161,76 @@
       </c>
       <c r="B102" s="15" t="inlineStr">
         <is>
+          <t>ai_technique</t>
+        </is>
+      </c>
+      <c r="C102" s="15" t="inlineStr">
+        <is>
+          <t>Technique Used</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="13.5" customFormat="1" customHeight="1" s="19">
+      <c r="A103" s="15" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B103" s="15" t="inlineStr">
+        <is>
           <t>semen_batch_number</t>
         </is>
       </c>
-      <c r="C102" s="15" t="inlineStr">
+      <c r="C103" s="15" t="inlineStr">
         <is>
           <t>Semen Batch Number</t>
         </is>
       </c>
-      <c r="D102" s="15" t="n"/>
-      <c r="E102" s="15" t="n"/>
-      <c r="F102" s="15" t="n"/>
-      <c r="G102" s="15" t="n"/>
-      <c r="H102" s="15" t="n"/>
-      <c r="I102" s="15" t="n"/>
-      <c r="J102" s="15" t="n"/>
-      <c r="K102" s="15" t="n"/>
-      <c r="L102" s="15" t="n"/>
-      <c r="M102" s="15" t="n"/>
-    </row>
-    <row r="103" ht="13.5" customFormat="1" customHeight="1" s="19">
-      <c r="A103" s="19" t="inlineStr">
-        <is>
-          <t>end_group</t>
-        </is>
-      </c>
+      <c r="D103" s="15" t="n"/>
+      <c r="E103" s="15" t="n"/>
+      <c r="F103" s="15" t="n"/>
+      <c r="G103" s="15" t="n"/>
+      <c r="H103" s="15" t="n"/>
+      <c r="I103" s="15" t="n"/>
+      <c r="J103" s="15" t="n"/>
+      <c r="K103" s="15" t="n"/>
+      <c r="L103" s="15" t="n"/>
+      <c r="M103" s="15" t="n"/>
     </row>
     <row r="104" ht="13.5" customFormat="1" customHeight="1" s="19">
       <c r="A104" s="19" t="inlineStr">
         <is>
+          <t>end_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="13.5" customFormat="1" customHeight="1" s="19">
+      <c r="A105" s="19" t="inlineStr">
+        <is>
           <t>end_repeat</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="13.5" customFormat="1" customHeight="1" s="19"/>
-    <row r="106" ht="13.5" customHeight="1" s="18">
-      <c r="A106" s="19" t="inlineStr">
+    <row r="106" ht="13.5" customHeight="1" s="18"/>
+    <row r="107" ht="13.5" customHeight="1" s="18">
+      <c r="A107" s="19" t="inlineStr">
         <is>
           <t>end_repeat</t>
         </is>
       </c>
-      <c r="B106" s="19" t="n"/>
-      <c r="C106" s="19" t="n"/>
-      <c r="D106" s="19" t="n"/>
-      <c r="E106" s="19" t="n"/>
-      <c r="F106" s="19" t="n"/>
-      <c r="G106" s="19" t="n"/>
-      <c r="H106" s="19" t="n"/>
-      <c r="I106" s="19" t="n"/>
-      <c r="J106" s="19" t="n"/>
-      <c r="K106" s="19" t="n"/>
-      <c r="L106" s="19" t="n"/>
-      <c r="M106" s="19" t="n"/>
-    </row>
-    <row r="107" ht="13.5" customHeight="1" s="18"/>
+      <c r="B107" s="19" t="n"/>
+      <c r="C107" s="19" t="n"/>
+      <c r="D107" s="19" t="n"/>
+      <c r="E107" s="19" t="n"/>
+      <c r="F107" s="19" t="n"/>
+      <c r="G107" s="19" t="n"/>
+      <c r="H107" s="19" t="n"/>
+      <c r="I107" s="19" t="n"/>
+      <c r="J107" s="19" t="n"/>
+      <c r="K107" s="19" t="n"/>
+      <c r="L107" s="19" t="n"/>
+      <c r="M107" s="19" t="n"/>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -6238,7 +6254,7 @@
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>v6</t>
+          <t>v7</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">

</xml_diff>